<commit_message>
Adding the court-room section
</commit_message>
<xml_diff>
--- a/case_priority_system/case_results.xlsx
+++ b/case_priority_system/case_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="92">
   <si>
     <t>Case_File</t>
   </si>
@@ -106,7 +106,7 @@
     <t>Accused, Complainant, Victim — names not disclosed</t>
   </si>
   <si>
-    <t>Pooja Exporters, Assistant Director, D.R.I.</t>
+    <t>Pooja Exporters vs Assistant Director, D.R.I</t>
   </si>
   <si>
     <t>The parties, AI, are involved in a legal dispute. The document indicates assault, victim, sexual assault, human trafficking. This case is classified as Criminal/Violent because the record matches assault, victim, sexual assault, human trafficking. Under the Constitution of India, the primary rights engaged are Article 21, Article 22, Article 20.</t>
@@ -121,7 +121,7 @@
     <t>The parties, Accused, Complainant, Victim — names not disclosed, are involved in a legal dispute. The document indicates assault, victim, sexual assault. This case is classified as Criminal/Violent because the record matches assault, victim, sexual assault. Under the Constitution of India, the primary rights engaged are Article 21, Article 22, Article 20.</t>
   </si>
   <si>
-    <t>The dispute is between Pooja Exporters and the Assistant Director, D.R.I. regarding an import licence for certain materials. The parties are arguing over conditions attached to the licence under the Imports (Control) Order, 1955. Pooja Exporters seeks clarification on the conditions of their import license while the D.R.I. is enforcing these conditions. This case falls under the Customs/Import-Export category as it deals with customs regulations and licences.</t>
+    <t>The parties, Pooja Exporters vs Assistant Director, D.R.I, are involved in a legal dispute. The document indicates customs, import, export, advance licence, d.r.i. This case is classified as Customs/Import-Export because the record matches customs, import, export, advance licence, d.r.i. Under the Constitution of India, the primary rights engaged are Article 14, Article 19(1)(g), Article 300A.</t>
   </si>
   <si>
     <t>## STATE'S CONSTITUTIONAL ASSESSMENT
@@ -348,9 +348,9 @@
 (Neutral, Unbiased Analysis from the Perspective of the Judiciary)
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
-**Parties:** Pooja Exporters, Assistant Director, D.R.I.
+**Parties:** Pooja Exporters vs Assistant Director, D.R.I
 **Legal Category:** Customs/Import-Export
-**Brief Description:** The dispute is between Pooja Exporters and the Assistant Director, D.R.I. regarding an import licence for certain materials. The parties are arguing over conditions attached to the licence under the Imports (Control) Order, 1955. Pooja Exporters seeks clarification on the conditions of their import license while the D.R.I. is enforcing these conditions. This case falls under the Customs/Import-Export category as it deals with customs regulations and licences.
+**Brief Description:** The parties, Pooja Exporters vs Assistant Director, D.R.I, are involved in a legal dispute. The document indicates customs, import, export, advance licence, d.r.i. This case is classified as Customs/Import-Export because the record matches customs, import, export, advance licence, d.r.i. Under the Constitution of India, the primary rights engaged are Article 14, Article 19(1)(g), Article 300A.
 **Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
 ### II. CONSTITUTIONAL RIGHTS ENGAGED
 The following constitutional provisions are relevant to this matter:
@@ -564,6 +564,9 @@
   </si>
   <si>
     <t>ANV-2026-0002</t>
+  </si>
+  <si>
+    <t>ANV-2026-0003</t>
   </si>
   <si>
     <t>FIR</t>
@@ -1219,7 +1222,7 @@
         <v>88</v>
       </c>
       <c r="T5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1281,7 +1284,7 @@
         <v>88</v>
       </c>
       <c r="T6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1343,7 +1346,7 @@
         <v>88</v>
       </c>
       <c r="T7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1402,10 +1405,10 @@
         <v>87</v>
       </c>
       <c r="S8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="T8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add CLAUDE.md, courtroom data, and new case ANV-2026-0004 with updated decision graphs
🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/case_priority_system/case_results.xlsx
+++ b/case_priority_system/case_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="134">
   <si>
     <t>Case_File</t>
   </si>
@@ -76,108 +76,148 @@
     <t>Document_Type</t>
   </si>
   <si>
+    <t>_upload_test.pdf</t>
+  </si>
+  <si>
     <t>AI.pdf</t>
   </si>
   <si>
-    <t>_upload_test.pdf</t>
+    <t>Alembic_Glass_Industries_Ltd_vs_Union_Of_India_And_Ors_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>Alembic_Glass_Industries_Ltd_vs_Union_Of_India_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>Asha_Rubber_Industries_Bangalore_vs_Collector_Of_Central_Excise_Bangalore_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>A_K_Kaimal_vs_Sudarsen_Trading_Co_Ltd_And_Anr_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>B_S_Madhva_Company_And_Ors_vs_Kapila_Textile_Mills_Ltd_And_Anr_on_1_January_1800.PDF</t>
   </si>
   <si>
     <t>Cipla_Limited_vs_Union_Of_India_on_1_January_1800.PDF</t>
   </si>
   <si>
+    <t>Deepak_Extrusion_And_Anr_vs_J_T_Chopra_Assistant_Collector_Of_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>Fictional_Case_Report_Test.pdf</t>
+  </si>
+  <si>
+    <t>Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>Rakhra_Sports_Private_Ltd_And_Others_vs_Khraitilal_Rakhra_And_Others_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>Sample_FIR_Case_Report_Sexual_Assault.pdf</t>
+  </si>
+  <si>
     <t>Sample_Medium_Priority_FIR.pdf</t>
   </si>
   <si>
-    <t>Sample_FIR_Case_Report_Sexual_Assault.pdf</t>
-  </si>
-  <si>
-    <t>Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800.PDF</t>
-  </si>
-  <si>
-    <t>AI</t>
+    <t>State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>_test_judgment.pdf</t>
   </si>
   <si>
     <t>Cipla Limited vs Union Of India</t>
   </si>
   <si>
-    <t>Sample Medium Priority FIR</t>
-  </si>
-  <si>
-    <t>Accused, Complainant, Victim — names not disclosed</t>
-  </si>
-  <si>
-    <t>Pooja Exporters vs Assistant Director, D.R.I</t>
-  </si>
-  <si>
-    <t>The parties, AI, are involved in a legal dispute. The document indicates assault, victim, sexual assault, human trafficking. This case is classified as Criminal/Violent because the record matches assault, victim, sexual assault, human trafficking. Under the Constitution of India, the primary rights engaged are Article 21, Article 22, Article 20.</t>
+    <t>AI-Powered Case Priority Prediction System, Judicial Authorities</t>
+  </si>
+  <si>
+    <t>Alembic Glass Industries Ltd, Union of India, Ors.</t>
+  </si>
+  <si>
+    <t>Alembic Glass Industries Ltd., Union of India</t>
+  </si>
+  <si>
+    <t>Asha Rubber Industries, Bangalore, Collector of Central Excise, Bangalore</t>
+  </si>
+  <si>
+    <t>A.K. Kaimal, Sudarsen Trading Co. Ltd. And Anr.</t>
+  </si>
+  <si>
+    <t>B.S. Madhva &amp; Company And Ors., Kapila Textile Mills Ltd., Bank of Mysore</t>
+  </si>
+  <si>
+    <t>Cipla Limited, Union of India</t>
+  </si>
+  <si>
+    <t>Deepak Extrusion And Anr., J.T. Chopra Assistant Collector Of ...</t>
+  </si>
+  <si>
+    <t>Emma Carter, Two Unidentified Males</t>
+  </si>
+  <si>
+    <t>Pooja Exporters, Assistant Director, D.R.I.</t>
+  </si>
+  <si>
+    <t>Rakhra Sports Private Ltd. And Others, Khraitilal Rakhra And Others</t>
+  </si>
+  <si>
+    <t>Complainant, Victim, Accused</t>
+  </si>
+  <si>
+    <t>Mr. Arun Kumar, Unknown</t>
+  </si>
+  <si>
+    <t>State of Karnataka, Union of India, Mysore Government Soap Factory, Mysore Sales International, Zonal Agents</t>
+  </si>
+  <si>
+    <t>Sanjay Kumar, S/O Naresh Prasad, The State of Bihar through Principal Secretary Department of Excise and Prohibition, Government of Bihar, Patna, The District Magistrate Cum Collector, Nawada, The Senior Superintendent of Police, Nawada, The Superintendent of Police, Excise and Prohibition, Nawada, The Office in Charge, Kauakol Police Station, Nawada</t>
   </si>
   <si>
     <t>The parties, Cipla Limited vs Union Of India, are involved in a legal dispute. The document indicates central excise, excise duty, collector of central excise, classification list, elt. This case is classified as Excise/Tax because the record matches central excise, excise duty, collector of central excise, classification list, elt. Under the Constitution of India, the primary rights engaged are Article 265, Article 14, Article 19(1)(g).</t>
   </si>
   <si>
-    <t>The parties, Sample Medium Priority FIR, are involved in a legal dispute. The document indicates property, charge. This case is classified as Property/Land because the record matches property, charge. Under the Constitution of India, the primary rights engaged are Article 300A, Article 14, Article 21.</t>
-  </si>
-  <si>
-    <t>The parties, Accused, Complainant, Victim — names not disclosed, are involved in a legal dispute. The document indicates assault, victim, sexual assault. This case is classified as Criminal/Violent because the record matches assault, victim, sexual assault. Under the Constitution of India, the primary rights engaged are Article 21, Article 22, Article 20.</t>
-  </si>
-  <si>
-    <t>The parties, Pooja Exporters vs Assistant Director, D.R.I, are involved in a legal dispute. The document indicates customs, import, export, advance licence, d.r.i. This case is classified as Customs/Import-Export because the record matches customs, import, export, advance licence, d.r.i. Under the Constitution of India, the primary rights engaged are Article 14, Article 19(1)(g), Article 300A.</t>
-  </si>
-  <si>
-    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
-(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
-This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
-### I. SUBJECT MATTER
-**Parties:** AI
-**Legal Category:** Criminal/Violent
-**Brief Description:** The parties, AI, are involved in a legal dispute. The document indicates assault, victim, sexual assault, human trafficking. This case is classified as Criminal/Violent because the record matches assault, victim, sexual assault, human trafficking. Under the Constitution of India, the primary rights engaged are Article 21, Article 22, Article 20.
-**Extracted Parameters:** Severity = Major, Vulnerability = High, Influence/ Power Imbalance = High
-### II. CONSTITUTIONAL RIGHTS ENGAGED
-The following constitutional provisions are relevant to this matter:
-- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
-  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
-- ****[PRIMARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
-  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
-- ****[PRIMARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
-  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
-- ****[SECONDARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
-  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
-- ****[SECONDARY]** Article 17 — Abolition of Untouchability**: Untouchability is abolished and its practice in any form is forbidden. The enforcement of any disability arising out of untouchability shall be an offence punishable in accordance with law.
-  - Key principles: Abolition of untouchability, Enforcement of disabilities is an offence, Protection of SC/ST communities
-- ****[SECONDARY]** Article 23 — Prohibition of Traffic in Human Beings and Forced Labour**: Traffic in human beings and begar and other similar forms of forced labour are prohibited. Any contravention of this provision shall be an offence punishable in accordance with law.
-  - Key principles: Prohibition of human trafficking, Prohibition of forced labour and begar
-- ****[SECONDARY]** Article 24 — Prohibition of Employment of Children in Factories**: No child below the age of fourteen years shall be employed to work in any factory or mine or engaged in any other hazardous employment.
-  - Key principles: No child labour below 14 in hazardous work, Protection of children from exploitation
-- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
-  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
-### III. SEVERITY &amp; URGENCY ASSESSMENT
-**Primary Article:** Article 21
-**Analysis:** The right to life under Article 21 includes the right to live with dignity and the right to health. Major injuries — especially those requiring hospitalisation, causing permanent disability, or posing life-threatening complications — constitute a serious interference with personal liberty and bodily integrity. The State must ensure prompt access to medical care, investigation of the incident, and accountability. Each day of delay risks permanent aggravation of the harm.
-**Urgency Classification:** High — bodily integrity and dignity are seriously compromised.
-### IV. STATE'S DUTY UNDER THE CONSTITUTION
-The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.
-### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
-**Vulnerability Level:** High
-This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
-**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
-**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
-**Influence Level:** High
-Government bodies, large corporations, regulatory authorities, or politically powerful individuals
-**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
-**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
-### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
-- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
-  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
-- **Doctrine of Parens Patriae**: The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.
-  - Application to this case: Critical for cases involving vulnerable victims — the state must act as guardian.
-- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
-  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
-### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
-**Assigned Priority:** High
-**Category Rationale:** Cases involving violent crime directly implicate the most fundamental right under the Constitution — the right to life. The state's failure to accord such cases the highest priority would constitute a violation of its affirmative obligation under Article 21 to protect life and ensure access to justice.
-### VIII. FINAL OBSERVATION
-From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **High Priority**. 
-This is constitutionally appropriate and reflects the gravity of the rights engaged. The court is directed to list this matter expeditiously, ensuring that no procedural delay undermines the constitutional rights at stake. The State must accord this case the attention and resources commensurate with its priority level.</t>
+    <t>The AI-Powered Case Priority Prediction System disputes the validity of the hybrid architecture and the use of large language models in making final decisions. The system argues that the hybrid approach is not transparent and does not align with constitutional principles. The case involves a dispute over the use of LLMs in judicial triage, engaging Article 14 (Equality Before Law) and Article 21 (Right to Life).</t>
+  </si>
+  <si>
+    <t>Alembic Glass Industries Ltd challenged the Union of India's demand for excise duty on packing charges of glassware. The Company argued that packing charges are not part of the excisable value and should not be taxed. The case involves a dispute over the classification of excisable goods under the Central Excises and Salt Act, 1944, and the constitutional right to protection of life and personal liberty (Article 21). The case falls under the Excise/Tax category as it deals with the levy and collection of excise duty on glassware packaging.</t>
+  </si>
+  <si>
+    <t>Alembic Glass Industries Ltd. filed a writ petition challenging the Assistant Collector of Central Excise's order granting a refund of excise duty. The dispute centers around the inclusion of the cost of packing materials supplied by buyers in the value of excisable goods for excise duty purposes. The petitioner argues that the cost of packing materials should not be included, while the respondent contends that the cost is deductible. The case involves constitutional and legal questions regarding the validity of Section 4(4)(d)(i) of the Central Excise and Salt Act, 1944. The case falls under the Excise/Tax category as it deals with excise duty and refund issues.</t>
+  </si>
+  <si>
+    <t>Asha Rubber Industries, Bangalore is contesting an order from the Collector of Central Excise, Bangalore regarding excise duty. The petitioner argues that the Collector's decision was based on unchallenged statements and reports, without giving the petitioner a chance to cross-examine. The case involves a dispute over the calculation of differential duty and the petitioner seeks dispensing with the pre-deposit of duty and penalty. The case falls under Excise/Tax as it deals with excise duty and related issues under the Central Excise Act.</t>
+  </si>
+  <si>
+    <t>In this case, A.K. Kaimal sought to be adjudged as an insolvent due to his inability to pay two debts. The appellant, A.K. Kaimal, approached the court to be declared insolvent, as he could not pay two items of debts due to the respondents. The court dismissed the petition, as the appellant had received a sum of Rs. 6,000 to 7,000 as a retirement benefit and could not account for its use. The case falls under the Insolvency/Debt category as it deals with the debtor's inability to pay debts, engaging Article 14 of the Indian Constitution, which prohibits discrimination and ensures equal protection.</t>
+  </si>
+  <si>
+    <t>This case involves a dispute between B.S. Madhva &amp; Company and Kapila Textile Mills Ltd. regarding the enforcement of an arbitration award and the priority of payments. The Bank of Mysore is a secured creditor. The case centers on the liquidation of Kapila Textile Mills Ltd. and the rights of the applicants (B.S. Madhva &amp; Company) to priority payment over other creditors. The case falls under the Company/Winding Up category as it deals with the winding up of a company and the rights of creditors and the liquidator.</t>
+  </si>
+  <si>
+    <t>Cipla Limited, a pharmaceutical company, challenged the classification of a chemical intermediate (BMS) as excisable under the Central Excise Act. The company argued that BMS is not a marketable commodity and should not be taxed, while the Union of India maintained that BMS is an excisable product. The case involves the interpretation of the Central Excise Act and the marketability test for excise duty. The constitutional article engaged is Article 14, as the case deals with the State's power imbalance and discrimination in tax classification.</t>
+  </si>
+  <si>
+    <t>The petitioners, Deepak Extrusion And Anr., challenge the constitutional validity of the amendment to Section 2(f) and Tariff Item 27 of the Central Excise Act. The case involves the levy of excise duty on aluminium containers that have been lacquered or printed. The Department argues that lacquering and printing are also a form of manufacture, while the petitioners contend that these processes are ancillary to the manufacture of the final product. The case raises questions about the scope of the term 'manufacture' in the Excise Act and the applicability of the decision in Empire Industries Ltd. v. Union of India to aluminium products.</t>
+  </si>
+  <si>
+    <t>Emma Carter, a store manager, was seriously injured during an armed robbery at a convenience store. Two unidentified males, one armed with a handgun and the other with a metal crowbar, assaulted her and stole cash and merchandise. The victim was hospitalized in ICU. The case involves serious physical harm and the potential for permanent disability, engaging Article 21 of the Constitution of India.</t>
+  </si>
+  <si>
+    <t>Pooja Exporters, a registered partnership firm, sought a writ of mandamus and prohibition against the Assistant Director, D.R.I. to release 51 bales of 100% mulberry raw silk seized by customs authorities. The petitioner argued that the seizure was illegal and in violation of their import licence, while the respondents contended that the petitioner had violated the actual user condition of the licence. The case falls under the Customs/Import-Export category as it involves customs seizure and import licence issues.</t>
+  </si>
+  <si>
+    <t>The dispute involves Rakhra Sports Private Ltd. and its directors, Khraitilal Rakhra and others, over the winding up of the company due to disagreements regarding the management and control of the business. The petitioners seek to have the company wound up under the Companies Act, alleging loss of mutual trust and exclusion from management. The case engages Article 14 of the Indian Constitution, as the petitioners assert the loss of their rights and the company's winding up unfairly prejudices their interests.</t>
+  </si>
+  <si>
+    <t>The complainant reports that the victim, a female aged [Age], was subjected to a sexual assault without her consent. The incident occurred at [Location] on [Date &amp; Time]. The victim informed a trusted individual and the matter was brought before the police. The complainant requests the investigation of the allegations, appropriate medical care, and legal action against the accused if the allegations are substantiated. This case falls under the Criminal/Violent category as it involves a serious assault on a vulnerable female victim.</t>
+  </si>
+  <si>
+    <t>Mr. Arun Kumar reported that his backpack, laptop, and accessories were stolen from a parked motorcycle. The theft occurred in the Market Road Parking Area. The case involves property damage and loss, as no physical injuries were reported. The investigation is ongoing, and the complainant seeks compensation for the loss. This case falls under General Civil as it deals with a property-related dispute and does not involve any immediate threat to life or ongoing violent incident.</t>
+  </si>
+  <si>
+    <t>The State of Karnataka petitioned against the Union of India and the Mysore Government Soap Factory over excise duty and tax issues. The factory manufactures soap and sells it through a sole agent and zonal agents. The dispute centers around the trade discount allowed on the wholesale price of the soap. The State of Karnataka seeks to have the wholesale cash price of the soap determined without the 6% trade discount, arguing that the discount should only apply to the sales made to the retail dealers and approved buyers at the factory premises. The case involves constitutional issues related to the right to profession and the right to move the Supreme Court for enforcement of fundamental rights (Article 226).</t>
+  </si>
+  <si>
+    <t>The case involves a writ petition seeking the release of a motorcycle seized by the police under the Bihar Prohibition and Excise Act. The petitioner, Sanjay Kumar, seeks the release of his motorcycle, which was seized in connection with a case registered under Section 30(a) of the Act. The case falls under the Excise/Tax category as it deals with the confiscation of property under the Bihar Prohibition and Excise Act, engaging Article 14 for the power imbalance and Article 21 for the protection of life and personal liberty.</t>
   </si>
   <si>
     <t>## STATE'S CONSTITUTIONAL ASSESSMENT
@@ -238,30 +278,86 @@
 (Neutral, Unbiased Analysis from the Perspective of the Judiciary)
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
-**Parties:** Sample Medium Priority FIR
-**Legal Category:** Property/Land
-**Brief Description:** The parties, Sample Medium Priority FIR, are involved in a legal dispute. The document indicates property, charge. This case is classified as Property/Land because the record matches property, charge. Under the Constitution of India, the primary rights engaged are Article 300A, Article 14, Article 21.
+**Parties:** AI-Powered Case Priority Prediction System, Judicial Authorities
+**Legal Category:** Criminal/Violent
+**Brief Description:** The AI-Powered Case Priority Prediction System disputes the validity of the hybrid architecture and the use of large language models in making final decisions. The system argues that the hybrid approach is not transparent and does not align with constitutional principles. The case involves a dispute over the use of LLMs in judicial triage, engaging Article 14 (Equality Before Law) and Article 21 (Right to Life).
+**Extracted Parameters:** Severity = Major, Vulnerability = High, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[PRIMARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[PRIMARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[SECONDARY]** Article 17 — Abolition of Untouchability**: Untouchability is abolished and its practice in any form is forbidden. The enforcement of any disability arising out of untouchability shall be an offence punishable in accordance with law.
+  - Key principles: Abolition of untouchability, Enforcement of disabilities is an offence, Protection of SC/ST communities
+- ****[SECONDARY]** Article 23 — Prohibition of Traffic in Human Beings and Forced Labour**: Traffic in human beings and begar and other similar forms of forced labour are prohibited. Any contravention of this provision shall be an offence punishable in accordance with law.
+  - Key principles: Prohibition of human trafficking, Prohibition of forced labour and begar
+- ****[SECONDARY]** Article 24 — Prohibition of Employment of Children in Factories**: No child below the age of fourteen years shall be employed to work in any factory or mine or engaged in any other hazardous employment.
+  - Key principles: No child labour below 14 in hazardous work, Protection of children from exploitation
+- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
+  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 21
+**Analysis:** The right to life under Article 21 includes the right to live with dignity and the right to health. Major injuries — especially those requiring hospitalisation, causing permanent disability, or posing life-threatening complications — constitute a serious interference with personal liberty and bodily integrity. The State must ensure prompt access to medical care, investigation of the incident, and accountability. Each day of delay risks permanent aggravation of the harm.
+**Urgency Classification:** High — bodily integrity and dignity are seriously compromised.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** High
+This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
+**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
+**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Doctrine of Parens Patriae**: The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.
+  - Application to this case: Critical for cases involving vulnerable victims — the state must act as guardian.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** High
+**Category Rationale:** Cases involving violent crime directly implicate the most fundamental right under the Constitution — the right to life. The state's failure to accord such cases the highest priority would constitute a violation of its affirmative obligation under Article 21 to protect life and ensure access to justice.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **High Priority**. 
+This is constitutionally appropriate and reflects the gravity of the rights engaged. The court is directed to list this matter expeditiously, ensuring that no procedural delay undermines the constitutional rights at stake. The State must accord this case the attention and resources commensurate with its priority level.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Alembic Glass Industries Ltd, Union of India, Ors.
+**Legal Category:** Excise/Tax
+**Brief Description:** Alembic Glass Industries Ltd challenged the Union of India's demand for excise duty on packing charges of glassware. The Company argued that packing charges are not part of the excisable value and should not be taxed. The case involves a dispute over the classification of excisable goods under the Central Excises and Salt Act, 1944, and the constitutional right to protection of life and personal liberty (Article 21). The case falls under the Excise/Tax category as it deals with the levy and collection of excise duty on glassware packaging.
 **Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
 ### II. CONSTITUTIONAL RIGHTS ENGAGED
 The following constitutional provisions are relevant to this matter:
-- ****[PRIMARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
-  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
 - ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
   - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
-- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
   - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
-- ****[SECONDARY]** Article 39 — Certain Principles of Policy to be Followed by the State**: The State shall direct its policy towards securing equal rights to an adequate means of livelihood, and that the ownership and control of material resources are so distributed as best to subserve the common good.
-  - Key principles: Adequate means of livelihood, Distribution of material resources for common good, Prevention of concentration of wealth, Protection of workers, children and women
-- ****[SECONDARY]** Article 46 — Promotion of Educational and Economic Interests of Weaker Sections**: The State shall promote with special care the educational and economic interests of the weaker sections of the people, and in particular of the Scheduled Castes and Scheduled Tribes, and shall protect them from social injustice and all forms of exploitation.
-  - Key principles: Special care for weaker sections, Protection of SC/ST from social injustice and exploitation
-- ****[SECONDARY]** Article 243G — Powers and Responsibilities of Panchayats**: The State legislature may endow Panchayats with such powers and authority as may be necessary to enable them to function as institutions of self-government, including in matters of land, water, agriculture and rural development.
-  - Key principles: Local self-government, Panchayat powers over land, water, agriculture
 ### III. SEVERITY &amp; URGENCY ASSESSMENT
 **Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
 **Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
 **Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
 ### IV. STATE'S DUTY UNDER THE CONSTITUTION
-Under Article 300A, no person shall be deprived of property except by authority of law. The State must ensure that land acquisition, eviction, and possession proceedings follow due process. When land disputes involve the homeless, tenants, or agricultural labourers, the right to livelihood under Article 21 is also engaged, requiring heightened judicial protection.
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
 ### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
 **Vulnerability Level:** Low
 This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
@@ -276,13 +372,13 @@
   - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
 - **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
   - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
-- **Doctrine of Legitimate Expectation**: A person who has a legitimate expectation based on a promise, practice or policy of the State is entitled to procedural fairness before that expectation is defeated.
-  - Application to this case: Applicable where administrative decisions frustrate settled practices, licences, or policies.
 - **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
   - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
 ### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
 **Assigned Priority:** Medium
-**Category Rationale:** Property and land disputes primarily affect economic and possessory rights. However, when they involve the right to shelter or livelihood (Article 21), priority should be elevated. Routine property disputes without violence or immediate displacement risk warrant standard queue processing.
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
 ### VIII. FINAL OBSERVATION
 From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
 The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
@@ -292,9 +388,333 @@
 (Neutral, Unbiased Analysis from the Perspective of the Judiciary)
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
-**Parties:** Accused, Complainant, Victim — names not disclosed
+**Parties:** Alembic Glass Industries Ltd., Union of India
+**Legal Category:** Excise/Tax
+**Brief Description:** Alembic Glass Industries Ltd. filed a writ petition challenging the Assistant Collector of Central Excise's order granting a refund of excise duty. The dispute centers around the inclusion of the cost of packing materials supplied by buyers in the value of excisable goods for excise duty purposes. The petitioner argues that the cost of packing materials should not be included, while the respondent contends that the cost is deductible. The case involves constitutional and legal questions regarding the validity of Section 4(4)(d)(i) of the Central Excise and Salt Act, 1944. The case falls under the Excise/Tax category as it deals with excise duty and refund issues.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Asha Rubber Industries, Bangalore, Collector of Central Excise, Bangalore
+**Legal Category:** Excise/Tax
+**Brief Description:** Asha Rubber Industries, Bangalore is contesting an order from the Collector of Central Excise, Bangalore regarding excise duty. The petitioner argues that the Collector's decision was based on unchallenged statements and reports, without giving the petitioner a chance to cross-examine. The case involves a dispute over the calculation of differential duty and the petitioner seeks dispensing with the pre-deposit of duty and penalty. The case falls under Excise/Tax as it deals with excise duty and related issues under the Central Excise Act.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** A.K. Kaimal, Sudarsen Trading Co. Ltd. And Anr.
+**Legal Category:** Excise/Tax
+**Brief Description:** In this case, A.K. Kaimal sought to be adjudged as an insolvent due to his inability to pay two debts. The appellant, A.K. Kaimal, approached the court to be declared insolvent, as he could not pay two items of debts due to the respondents. The court dismissed the petition, as the appellant had received a sum of Rs. 6,000 to 7,000 as a retirement benefit and could not account for its use. The case falls under the Insolvency/Debt category as it deals with the debtor's inability to pay debts, engaging Article 14 of the Indian Constitution, which prohibits discrimination and ensures equal protection.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = Low
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** Low
+Individuals, small businesses, or parties of comparable standing
+**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
+**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Low
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Low Priority**. 
+No urgent constitutional concern is identified. The matter should proceed in regular course. The court remains obligated under Article 14 to ensure that this matter is adjudicated fairly and without inordinate delay, even if it does not warrant special expedition.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** B.S. Madhva &amp; Company And Ors., Kapila Textile Mills Ltd., Bank of Mysore
+**Legal Category:** Excise/Tax
+**Brief Description:** This case involves a dispute between B.S. Madhva &amp; Company and Kapila Textile Mills Ltd. regarding the enforcement of an arbitration award and the priority of payments. The Bank of Mysore is a secured creditor. The case centers on the liquidation of Kapila Textile Mills Ltd. and the rights of the applicants (B.S. Madhva &amp; Company) to priority payment over other creditors. The case falls under the Company/Winding Up category as it deals with the winding up of a company and the rights of creditors and the liquidator.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Cipla Limited, Union of India
+**Legal Category:** Excise/Tax
+**Brief Description:** Cipla Limited, a pharmaceutical company, challenged the classification of a chemical intermediate (BMS) as excisable under the Central Excise Act. The company argued that BMS is not a marketable commodity and should not be taxed, while the Union of India maintained that BMS is an excisable product. The case involves the interpretation of the Central Excise Act and the marketability test for excise duty. The constitutional article engaged is Article 14, as the case deals with the State's power imbalance and discrimination in tax classification.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Deepak Extrusion And Anr., J.T. Chopra Assistant Collector Of ...
+**Legal Category:** Excise/Tax
+**Brief Description:** The petitioners, Deepak Extrusion And Anr., challenge the constitutional validity of the amendment to Section 2(f) and Tariff Item 27 of the Central Excise Act. The case involves the levy of excise duty on aluminium containers that have been lacquered or printed. The Department argues that lacquering and printing are also a form of manufacture, while the petitioners contend that these processes are ancillary to the manufacture of the final product. The case raises questions about the scope of the term 'manufacture' in the Excise Act and the applicability of the decision in Empire Industries Ltd. v. Union of India to aluminium products.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Emma Carter, Two Unidentified Males
 **Legal Category:** Criminal/Violent
-**Brief Description:** The parties, Accused, Complainant, Victim — names not disclosed, are involved in a legal dispute. The document indicates assault, victim, sexual assault. This case is classified as Criminal/Violent because the record matches assault, victim, sexual assault. Under the Constitution of India, the primary rights engaged are Article 21, Article 22, Article 20.
+**Brief Description:** Emma Carter, a store manager, was seriously injured during an armed robbery at a convenience store. Two unidentified males, one armed with a handgun and the other with a metal crowbar, assaulted her and stole cash and merchandise. The victim was hospitalized in ICU. The case involves serious physical harm and the potential for permanent disability, engaging Article 21 of the Constitution of India.
 **Extracted Parameters:** Severity = Major, Vulnerability = High, Influence/ Power Imbalance = Low
 ### II. CONSTITUTIONAL RIGHTS ENGAGED
 The following constitutional provisions are relevant to this matter:
@@ -348,9 +768,9 @@
 (Neutral, Unbiased Analysis from the Perspective of the Judiciary)
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
-**Parties:** Pooja Exporters vs Assistant Director, D.R.I
+**Parties:** Pooja Exporters, Assistant Director, D.R.I.
 **Legal Category:** Customs/Import-Export
-**Brief Description:** The parties, Pooja Exporters vs Assistant Director, D.R.I, are involved in a legal dispute. The document indicates customs, import, export, advance licence, d.r.i. This case is classified as Customs/Import-Export because the record matches customs, import, export, advance licence, d.r.i. Under the Constitution of India, the primary rights engaged are Article 14, Article 19(1)(g), Article 300A.
+**Brief Description:** Pooja Exporters, a registered partnership firm, sought a writ of mandamus and prohibition against the Assistant Director, D.R.I. to release 51 bales of 100% mulberry raw silk seized by customs authorities. The petitioner argued that the seizure was illegal and in violation of their import licence, while the respondents contended that the petitioner had violated the actual user condition of the licence. The case falls under the Customs/Import-Export category as it involves customs seizure and import licence issues.
 **Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
 ### II. CONSTITUTIONAL RIGHTS ENGAGED
 The following constitutional provisions are relevant to this matter:
@@ -396,6 +816,282 @@
 The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
   </si>
   <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Rakhra Sports Private Ltd. And Others, Khraitilal Rakhra And Others
+**Legal Category:** Excise/Tax
+**Brief Description:** The dispute involves Rakhra Sports Private Ltd. and its directors, Khraitilal Rakhra and others, over the winding up of the company due to disagreements regarding the management and control of the business. The petitioners seek to have the company wound up under the Companies Act, alleging loss of mutual trust and exclusion from management. The case engages Article 14 of the Indian Constitution, as the petitioners assert the loss of their rights and the company's winding up unfairly prejudices their interests.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Complainant, Victim, Accused
+**Legal Category:** Criminal/Violent
+**Brief Description:** The complainant reports that the victim, a female aged [Age], was subjected to a sexual assault without her consent. The incident occurred at [Location] on [Date &amp; Time]. The victim informed a trusted individual and the matter was brought before the police. The complainant requests the investigation of the allegations, appropriate medical care, and legal action against the accused if the allegations are substantiated. This case falls under the Criminal/Violent category as it involves a serious assault on a vulnerable female victim.
+**Extracted Parameters:** Severity = Major, Vulnerability = High, Influence/ Power Imbalance = Low
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[PRIMARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[PRIMARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[SECONDARY]** Article 17 — Abolition of Untouchability**: Untouchability is abolished and its practice in any form is forbidden. The enforcement of any disability arising out of untouchability shall be an offence punishable in accordance with law.
+  - Key principles: Abolition of untouchability, Enforcement of disabilities is an offence, Protection of SC/ST communities
+- ****[SECONDARY]** Article 23 — Prohibition of Traffic in Human Beings and Forced Labour**: Traffic in human beings and begar and other similar forms of forced labour are prohibited. Any contravention of this provision shall be an offence punishable in accordance with law.
+  - Key principles: Prohibition of human trafficking, Prohibition of forced labour and begar
+- ****[SECONDARY]** Article 24 — Prohibition of Employment of Children in Factories**: No child below the age of fourteen years shall be employed to work in any factory or mine or engaged in any other hazardous employment.
+  - Key principles: No child labour below 14 in hazardous work, Protection of children from exploitation
+- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
+  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 21
+**Analysis:** The right to life under Article 21 includes the right to live with dignity and the right to health. Major injuries — especially those requiring hospitalisation, causing permanent disability, or posing life-threatening complications — constitute a serious interference with personal liberty and bodily integrity. The State must ensure prompt access to medical care, investigation of the incident, and accountability. Each day of delay risks permanent aggravation of the harm.
+**Urgency Classification:** High — bodily integrity and dignity are seriously compromised.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** High
+This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
+**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
+**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
+**Influence Level:** Low
+Individuals, small businesses, or parties of comparable standing
+**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
+**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Doctrine of Parens Patriae**: The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.
+  - Application to this case: Critical for cases involving vulnerable victims — the state must act as guardian.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** High
+**Category Rationale:** Cases involving violent crime directly implicate the most fundamental right under the Constitution — the right to life. The state's failure to accord such cases the highest priority would constitute a violation of its affirmative obligation under Article 21 to protect life and ensure access to justice.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **High Priority**. 
+This is constitutionally appropriate and reflects the gravity of the rights engaged. The court is directed to list this matter expeditiously, ensuring that no procedural delay undermines the constitutional rights at stake. The State must accord this case the attention and resources commensurate with its priority level.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Mr. Arun Kumar, Unknown
+**Legal Category:** Excise/Tax
+**Brief Description:** Mr. Arun Kumar reported that his backpack, laptop, and accessories were stolen from a parked motorcycle. The theft occurred in the Market Road Parking Area. The case involves property damage and loss, as no physical injuries were reported. The investigation is ongoing, and the complainant seeks compensation for the loss. This case falls under General Civil as it deals with a property-related dispute and does not involve any immediate threat to life or ongoing violent incident.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** State of Karnataka, Union of India, Mysore Government Soap Factory, Mysore Sales International, Zonal Agents
+**Legal Category:** Excise/Tax
+**Brief Description:** The State of Karnataka petitioned against the Union of India and the Mysore Government Soap Factory over excise duty and tax issues. The factory manufactures soap and sells it through a sole agent and zonal agents. The dispute centers around the trade discount allowed on the wholesale price of the soap. The State of Karnataka seeks to have the wholesale cash price of the soap determined without the 6% trade discount, arguing that the discount should only apply to the sales made to the retail dealers and approved buyers at the factory premises. The case involves constitutional issues related to the right to profession and the right to move the Supreme Court for enforcement of fundamental rights (Article 226).
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Sanjay Kumar, S/O Naresh Prasad, The State of Bihar through Principal Secretary Department of Excise and Prohibition, Government of Bihar, Patna, The District Magistrate Cum Collector, Nawada, The Senior Superintendent of Police, Nawada, The Superintendent of Police, Excise and Prohibition, Nawada, The Office in Charge, Kauakol Police Station, Nawada
+**Legal Category:** Customs/Import-Export
+**Brief Description:** The case involves a writ petition seeking the release of a motorcycle seized by the police under the Bihar Prohibition and Excise Act. The petitioner, Sanjay Kumar, seeks the release of his motorcycle, which was seized in connection with a case registered under Section 30(a) of the Act. The case falls under the Excise/Tax category as it deals with the confiscation of property under the Bihar Prohibition and Excise Act, engaging Article 14 for the power imbalance and Article 21 for the protection of life and personal liberty.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[PRIMARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State must ensure that customs and import-export regulations are enforced lawfully and proportionately. Seizures, confiscations, and penalties must have legal sanction and must not arbitrarily deprive a person of their right to trade (Article 19(1)(g)) or property (Article 300A). The Directorate of Revenue Intelligence and customs authorities must act within the bounds of the law.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Doctrine of Legitimate Expectation**: A person who has a legitimate expectation based on a promise, practice or policy of the State is entitled to procedural fairness before that expectation is defeated.
+  - Application to this case: Applicable where administrative decisions frustrate settled practices, licences, or policies.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Customs and trade matters primarily affect commercial and property rights. While procedural fairness is critical, these cases do not typically involve threats to life or physical safety. Priority should be based on the quantum of economic impact, with exceptional urgency only when perishable goods, personal liberty, or livelihood of vulnerable persons is at stake.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+  </si>
+  <si>
     <t>**RULE 1 — Major Injury → High Priority (Article 21):** Bodily integrity and the right to health under Article 21 are seriously compromised. Strong urgency is constitutionally required.
 **RULE 2 — High Vulnerability → Elevated Priority (Doctrine of Parens Patriae):** The state has a special duty to protect vulnerable persons. Articles 15, 39, and 39A require the court to ensure that vulnerable litigants are not disadvantaged by delay.
 **RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
@@ -404,15 +1100,8 @@
   </si>
   <si>
     <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
-**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
 **RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
-**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
-  </si>
-  <si>
-    <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
-**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
-**RULE 4 — Property/Land Dispute → Article 300A &amp; Livelihood:** Article 300A protects property rights. If livelihood (Article 21) is affected, priority should be elevated accordingly.
-**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Low**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
   </si>
   <si>
     <t>**RULE 1 — Major Injury → High Priority (Article 21):** Bodily integrity and the right to health under Article 21 are seriously compromised. Strong urgency is constitutionally required.
@@ -421,100 +1110,129 @@
 **FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **High**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
   </si>
   <si>
+    <t>case_priority_system/decision_graphs\upload_test_decision_report.md</t>
+  </si>
+  <si>
     <t>case_priority_system/decision_graphs\AI_decision_report.md</t>
   </si>
   <si>
-    <t>case_priority_system/decision_graphs\upload_test_decision_report.md</t>
+    <t>case_priority_system/decision_graphs\Alembic_Glass_Industries_Ltd_vs_Union_Of_India_And_Ors_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Alembic_Glass_Industries_Ltd_vs_Union_Of_India_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Asha_Rubber_Industries_Bangalore_vs_Collector_Of_Central_Excise_Bangalore_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\A_K_Kaimal_vs_Sudarsen_Trading_Co_Ltd_And_Anr_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\B_S_Madhva_Company_And_Ors_vs_Kapila_Textile_Mills_Ltd_And_Anr_on_1_January_1800_decision_report.md</t>
   </si>
   <si>
     <t>case_priority_system/decision_graphs\Cipla_Limited_vs_Union_Of_India_on_1_January_1800_decision_report.md</t>
   </si>
   <si>
+    <t>case_priority_system/decision_graphs\Deepak_Extrusion_And_Anr_vs_J_T_Chopra_Assistant_Collector_Of_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Fictional_Case_Report_Test_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Rakhra_Sports_Private_Ltd_And_Others_vs_Khraitilal_Rakhra_And_Others_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Sample_FIR_Case_Report_Sexual_Assault_decision_report.md</t>
+  </si>
+  <si>
     <t>case_priority_system/decision_graphs\Sample_Medium_Priority_FIR_decision_report.md</t>
   </si>
   <si>
-    <t>case_priority_system/decision_graphs\Sample_FIR_Case_Report_Sexual_Assault_decision_report.md</t>
-  </si>
-  <si>
-    <t>case_priority_system/decision_graphs\Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800_decision_report.md</t>
+    <t>case_priority_system/decision_graphs\State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\test_judgment_decision_report.md</t>
+  </si>
+  <si>
+    <t>Node 0: Severity is one of: Fatal, Major; case value = No Injury; result = No -&gt; Node 4: Influence / power imbalance is one of: High; case value = High; result = Yes -&gt; Leaf node 5 =&gt; Predicted Priority = Medium</t>
   </si>
   <si>
     <t>Node 0: Severity is one of: Fatal, Major; case value = Major; result = Yes -&gt; Node 1: Shri score &lt;= 0.0720; case value = 0.0000; result = Yes -&gt; Leaf node 2 =&gt; Predicted Priority = High</t>
   </si>
   <si>
-    <t>Node 0: Severity is one of: Fatal, Major; case value = No Injury; result = No -&gt; Node 4: Influence / power imbalance is one of: High; case value = High; result = Yes -&gt; Leaf node 5 =&gt; Predicted Priority = Medium</t>
+    <t>Node 0: Severity is one of: Fatal, Major; case value = No Injury; result = No -&gt; Node 4: Influence / power imbalance is one of: High; case value = Low; result = No -&gt; Node 6: Severity is one of: Fatal, Major, Minor; case value = No Injury; result = No -&gt; Node 8: Vulnerability is one of: High; case value = Low; result = No -&gt; Node 10: Legal category is one of: Company/Winding Up, Constitutional/Writ, Criminal/Violent, Customs/Import-Export, Excise/Tax, General Civil; case value = Excise/Tax; result = Yes -&gt; Node 11: Dispute Concerning score &lt;= 0.2136; case value = 0.0000; result = Yes -&gt; Leaf node 12 =&gt; Predicted Priority = Low</t>
+  </si>
+  <si>
+    <t>Medium</t>
   </si>
   <si>
     <t>High</t>
   </si>
   <si>
-    <t>Medium</t>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Excise/Tax</t>
   </si>
   <si>
     <t>Criminal/Violent</t>
   </si>
   <si>
-    <t>Excise/Tax</t>
-  </si>
-  <si>
-    <t>Property/Land</t>
-  </si>
-  <si>
     <t>Customs/Import-Export</t>
   </si>
   <si>
+    <t>Non-Violent</t>
+  </si>
+  <si>
     <t>Violent</t>
   </si>
   <si>
-    <t>Non-Violent</t>
-  </si>
-  <si>
-    <t>Property</t>
+    <t>No Injury</t>
   </si>
   <si>
     <t>Major</t>
   </si>
   <si>
-    <t>No Injury</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>[{'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': True}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': True}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': False}, {'article': 'Article 17', 'title': 'Abolition of Untouchability', 'primary': False}, {'article': 'Article 23', 'title': 'Prohibition of Traffic in Human Beings and Forced Labour', 'primary': False}, {'article': 'Article 24', 'title': 'Prohibition of Employment of Children in Factories', 'primary': False}, {'article': 'Article 39A', 'title': 'Equal Justice and Free Legal Aid', 'primary': False}]</t>
-  </si>
-  <si>
     <t>[{'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': True}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': False}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False}]</t>
   </si>
   <si>
-    <t>[{'article': 'Article 300A', 'title': 'Right to Property', 'primary': True}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True}, {'article': 'Article 39', 'title': 'Certain Principles of Policy to be Followed by the State', 'primary': False}, {'article': 'Article 46', 'title': 'Promotion of Educational and Economic Interests of Weaker Sections', 'primary': False}, {'article': 'Article 243G', 'title': 'Powers and Responsibilities of Panchayats', 'primary': False}]</t>
-  </si>
-  <si>
-    <t>[{'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': True}, {'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': False}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False}]</t>
+    <t>Article 21 (Primary), Article 22 (Primary), Article 20 (Primary), Article 14 (Secondary), Article 17 (Secondary), Article 23 (Secondary), Article 24 (Secondary), Article 39A (Secondary)</t>
+  </si>
+  <si>
+    <t>Article 265 (Primary), Article 14 (Primary), Article 19(1)(g) (Primary), Article 300A (Secondary), Article 301 (Secondary), Article 21 (Secondary)</t>
+  </si>
+  <si>
+    <t>Article 14 (Primary), Article 19(1)(g) (Primary), Article 300A (Primary), Article 265 (Secondary), Article 301 (Secondary), Article 21 (Secondary)</t>
+  </si>
+  <si>
+    <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
   </si>
   <si>
     <t>The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.</t>
   </si>
   <si>
-    <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
-  </si>
-  <si>
-    <t>Under Article 300A, no person shall be deprived of property except by authority of law. The State must ensure that land acquisition, eviction, and possession proceedings follow due process. When land disputes involve the homeless, tenants, or agricultural labourers, the right to livelihood under Article 21 is also engaged, requiring heightened judicial protection.</t>
-  </si>
-  <si>
     <t>The State must ensure that customs and import-export regulations are enforced lawfully and proportionately. Seizures, confiscations, and penalties must have legal sanction and must not arbitrarily deprive a person of their right to trade (Article 19(1)(g)) or property (Article 300A). The Directorate of Revenue Intelligence and customs authorities must act within the bounds of the law.</t>
   </si>
   <si>
-    <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Doctrine of Parens Patriae', 'description': 'The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.', 'application': 'Critical for cases involving vulnerable victims — the state must act as guardian.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}]</t>
-  </si>
-  <si>
     <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Reasonable Classification', 'description': 'Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.', 'application': 'Used to test whether differential treatment of litigants or groups is constitutional.'}]</t>
   </si>
   <si>
-    <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Doctrine of Legitimate Expectation', 'description': 'A person who has a legitimate expectation based on a promise, practice or policy of the State is entitled to procedural fairness before that expectation is defeated.', 'application': 'Applicable where administrative decisions frustrate settled practices, licences, or policies.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}]</t>
-  </si>
-  <si>
-    <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Doctrine of Legitimate Expectation', 'description': 'A person who has a legitimate expectation based on a promise, practice or policy of the State is entitled to procedural fairness before that expectation is defeated.', 'application': 'Applicable where administrative decisions frustrate settled practices, licences, or policies.'}]</t>
+    <t>Doctrine of Proportionality; Doctrine of Parens Patriae; Rule of Law</t>
+  </si>
+  <si>
+    <t>Doctrine of Proportionality; Principle of Natural Justice — Audi Alteram Partem; Rule of Law; Doctrine of Reasonable Classification</t>
+  </si>
+  <si>
+    <t>Doctrine of Proportionality; Principle of Natural Justice — Audi Alteram Partem; Doctrine of Legitimate Expectation</t>
+  </si>
+  <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
   </si>
   <si>
     <t>**Primary Interest — Right to Life &amp; Bodily Integrity (Article 21):** The severity level 'Major' indicates that the right to life or physical integrity has been seriously compromised. Under Article 21, this is the weightiest constitutional interest and must take precedence over all other considerations. The state's duty to protect life is non-derogable and non-delegable.
@@ -525,13 +1243,7 @@
   </si>
   <si>
     <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
-**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
 **Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
-  </si>
-  <si>
-    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
-**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
-**Category-Specific Analysis — Property/Land:** Property rights under Article 300A are constitutional but not absolute. The priority should consider whether the dispute involves livelihood (Article 21) or mere property entitlement.</t>
   </si>
   <si>
     <t>**Primary Interest — Right to Life &amp; Bodily Integrity (Article 21):** The severity level 'Major' indicates that the right to life or physical integrity has been seriously compromised. Under Article 21, this is the weightiest constitutional interest and must take precedence over all other considerations. The state's duty to protect life is non-derogable and non-delegable.
@@ -545,34 +1257,7 @@
 **Category-Specific Analysis — Customs/Import-Export:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
   </si>
   <si>
-    <t>case_priority_system\reports\AI_report.pdf</t>
-  </si>
-  <si>
     <t>case_priority_system\reports\_upload_test_report.pdf</t>
-  </si>
-  <si>
-    <t>case_priority_system\reports\Cipla_Limited_vs_Union_Of_India_on_1_January_1800_report.pdf</t>
-  </si>
-  <si>
-    <t>case_priority_system\reports\Sample_Medium_Priority_FIR_report.pdf</t>
-  </si>
-  <si>
-    <t>case_priority_system\reports\Sample_FIR_Case_Report_Sexual_Assault_report.pdf</t>
-  </si>
-  <si>
-    <t>case_priority_system\reports\Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800_report.pdf</t>
-  </si>
-  <si>
-    <t>ANV-2026-0002</t>
-  </si>
-  <si>
-    <t>ANV-2026-0003</t>
-  </si>
-  <si>
-    <t>FIR</t>
-  </si>
-  <si>
-    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -930,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1000,55 +1685,55 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="F2" t="s">
-        <v>45</v>
+        <v>88</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="H2" t="s">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="J2" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
       <c r="K2" t="s">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="L2" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="M2" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="N2" t="s">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="O2" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="P2" t="s">
-        <v>73</v>
+        <v>124</v>
       </c>
       <c r="Q2" t="s">
-        <v>77</v>
+        <v>128</v>
       </c>
       <c r="R2" t="s">
-        <v>82</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1056,55 +1741,52 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>89</v>
       </c>
       <c r="G3" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>108</v>
       </c>
       <c r="I3" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="J3" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="K3" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="L3" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="M3" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="N3" t="s">
-        <v>66</v>
+        <v>118</v>
       </c>
       <c r="O3" t="s">
-        <v>70</v>
+        <v>122</v>
       </c>
       <c r="P3" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
       <c r="Q3" t="s">
-        <v>78</v>
-      </c>
-      <c r="R3" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1112,55 +1794,52 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="G4" t="s">
-        <v>52</v>
+        <v>104</v>
       </c>
       <c r="H4" t="s">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="I4" t="s">
-        <v>56</v>
+        <v>110</v>
       </c>
       <c r="J4" t="s">
-        <v>60</v>
+        <v>113</v>
       </c>
       <c r="K4" t="s">
-        <v>63</v>
+        <v>115</v>
       </c>
       <c r="L4" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="M4" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="N4" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="O4" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="P4" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="Q4" t="s">
-        <v>78</v>
-      </c>
-      <c r="R4" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1168,61 +1847,52 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="G5" t="s">
-        <v>48</v>
+        <v>104</v>
       </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="I5" t="s">
-        <v>57</v>
+        <v>110</v>
       </c>
       <c r="J5" t="s">
-        <v>61</v>
+        <v>113</v>
       </c>
       <c r="K5" t="s">
-        <v>63</v>
+        <v>115</v>
       </c>
       <c r="L5" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="M5" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="N5" t="s">
-        <v>67</v>
+        <v>119</v>
       </c>
       <c r="O5" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="P5" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="Q5" t="s">
-        <v>79</v>
-      </c>
-      <c r="R5" t="s">
-        <v>85</v>
-      </c>
-      <c r="S5" t="s">
-        <v>88</v>
-      </c>
-      <c r="T5" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1230,185 +1900,635 @@
         <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="E6" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="F6" t="s">
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="G6" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="I6" t="s">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="J6" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
       <c r="K6" t="s">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="L6" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="M6" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="N6" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="O6" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="P6" t="s">
-        <v>73</v>
+        <v>126</v>
       </c>
       <c r="Q6" t="s">
-        <v>80</v>
-      </c>
-      <c r="R6" t="s">
-        <v>86</v>
-      </c>
-      <c r="S6" t="s">
-        <v>88</v>
-      </c>
-      <c r="T6" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="E7" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="F7" t="s">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="G7" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
       <c r="H7" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="J7" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
       <c r="K7" t="s">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="L7" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="M7" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="N7" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="O7" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="P7" t="s">
-        <v>73</v>
+        <v>126</v>
       </c>
       <c r="Q7" t="s">
-        <v>80</v>
-      </c>
-      <c r="R7" t="s">
-        <v>86</v>
-      </c>
-      <c r="S7" t="s">
-        <v>88</v>
-      </c>
-      <c r="T7" t="s">
-        <v>91</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G8" t="s">
+        <v>104</v>
+      </c>
+      <c r="H8" t="s">
+        <v>107</v>
+      </c>
+      <c r="I8" t="s">
+        <v>110</v>
+      </c>
+      <c r="J8" t="s">
+        <v>113</v>
+      </c>
+      <c r="K8" t="s">
+        <v>115</v>
+      </c>
+      <c r="L8" t="s">
+        <v>109</v>
+      </c>
+      <c r="M8" t="s">
+        <v>108</v>
+      </c>
+      <c r="N8" t="s">
+        <v>119</v>
+      </c>
+      <c r="O8" t="s">
+        <v>121</v>
+      </c>
+      <c r="P8" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" t="s">
+        <v>95</v>
+      </c>
+      <c r="G9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H9" t="s">
+        <v>107</v>
+      </c>
+      <c r="I9" t="s">
+        <v>110</v>
+      </c>
+      <c r="J9" t="s">
+        <v>113</v>
+      </c>
+      <c r="K9" t="s">
+        <v>115</v>
+      </c>
+      <c r="L9" t="s">
+        <v>109</v>
+      </c>
+      <c r="M9" t="s">
+        <v>108</v>
+      </c>
+      <c r="N9" t="s">
+        <v>119</v>
+      </c>
+      <c r="O9" t="s">
+        <v>121</v>
+      </c>
+      <c r="P9" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" t="s">
+        <v>96</v>
+      </c>
+      <c r="G10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H10" t="s">
+        <v>107</v>
+      </c>
+      <c r="I10" t="s">
+        <v>110</v>
+      </c>
+      <c r="J10" t="s">
+        <v>113</v>
+      </c>
+      <c r="K10" t="s">
+        <v>115</v>
+      </c>
+      <c r="L10" t="s">
+        <v>109</v>
+      </c>
+      <c r="M10" t="s">
+        <v>108</v>
+      </c>
+      <c r="N10" t="s">
+        <v>119</v>
+      </c>
+      <c r="O10" t="s">
+        <v>121</v>
+      </c>
+      <c r="P10" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F11" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" t="s">
+        <v>108</v>
+      </c>
+      <c r="I11" t="s">
+        <v>111</v>
+      </c>
+      <c r="J11" t="s">
+        <v>114</v>
+      </c>
+      <c r="K11" t="s">
+        <v>116</v>
+      </c>
+      <c r="L11" t="s">
+        <v>108</v>
+      </c>
+      <c r="M11" t="s">
+        <v>109</v>
+      </c>
+      <c r="N11" t="s">
+        <v>118</v>
+      </c>
+      <c r="O11" t="s">
+        <v>122</v>
+      </c>
+      <c r="P11" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20">
+      <c r="A12" t="s">
         <v>30</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" t="s">
+        <v>98</v>
+      </c>
+      <c r="G12" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" t="s">
+        <v>107</v>
+      </c>
+      <c r="I12" t="s">
+        <v>112</v>
+      </c>
+      <c r="J12" t="s">
+        <v>113</v>
+      </c>
+      <c r="K12" t="s">
+        <v>115</v>
+      </c>
+      <c r="L12" t="s">
+        <v>109</v>
+      </c>
+      <c r="M12" t="s">
+        <v>108</v>
+      </c>
+      <c r="N12" t="s">
+        <v>120</v>
+      </c>
+      <c r="O12" t="s">
+        <v>123</v>
+      </c>
+      <c r="P12" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G13" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" t="s">
+        <v>110</v>
+      </c>
+      <c r="J13" t="s">
+        <v>113</v>
+      </c>
+      <c r="K13" t="s">
+        <v>115</v>
+      </c>
+      <c r="L13" t="s">
+        <v>109</v>
+      </c>
+      <c r="M13" t="s">
+        <v>108</v>
+      </c>
+      <c r="N13" t="s">
+        <v>119</v>
+      </c>
+      <c r="O13" t="s">
+        <v>121</v>
+      </c>
+      <c r="P13" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" t="s">
+        <v>87</v>
+      </c>
+      <c r="F14" t="s">
+        <v>100</v>
+      </c>
+      <c r="G14" t="s">
+        <v>105</v>
+      </c>
+      <c r="H14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I14" t="s">
+        <v>111</v>
+      </c>
+      <c r="J14" t="s">
+        <v>114</v>
+      </c>
+      <c r="K14" t="s">
+        <v>116</v>
+      </c>
+      <c r="L14" t="s">
+        <v>108</v>
+      </c>
+      <c r="M14" t="s">
+        <v>109</v>
+      </c>
+      <c r="N14" t="s">
+        <v>118</v>
+      </c>
+      <c r="O14" t="s">
+        <v>122</v>
+      </c>
+      <c r="P14" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" t="s">
+        <v>101</v>
+      </c>
+      <c r="G15" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" t="s">
+        <v>107</v>
+      </c>
+      <c r="I15" t="s">
+        <v>110</v>
+      </c>
+      <c r="J15" t="s">
+        <v>113</v>
+      </c>
+      <c r="K15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L15" t="s">
+        <v>109</v>
+      </c>
+      <c r="M15" t="s">
+        <v>108</v>
+      </c>
+      <c r="N15" t="s">
+        <v>119</v>
+      </c>
+      <c r="O15" t="s">
+        <v>121</v>
+      </c>
+      <c r="P15" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" t="s">
+        <v>82</v>
+      </c>
+      <c r="E16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" t="s">
+        <v>102</v>
+      </c>
+      <c r="G16" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" t="s">
+        <v>107</v>
+      </c>
+      <c r="I16" t="s">
+        <v>110</v>
+      </c>
+      <c r="J16" t="s">
+        <v>113</v>
+      </c>
+      <c r="K16" t="s">
+        <v>115</v>
+      </c>
+      <c r="L16" t="s">
+        <v>109</v>
+      </c>
+      <c r="M16" t="s">
+        <v>108</v>
+      </c>
+      <c r="N16" t="s">
+        <v>119</v>
+      </c>
+      <c r="O16" t="s">
+        <v>121</v>
+      </c>
+      <c r="P16" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
+      <c r="A17" t="s">
         <v>35</v>
       </c>
-      <c r="D8" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" t="s">
-        <v>54</v>
-      </c>
-      <c r="I8" t="s">
-        <v>58</v>
-      </c>
-      <c r="J8" t="s">
-        <v>60</v>
-      </c>
-      <c r="K8" t="s">
-        <v>63</v>
-      </c>
-      <c r="L8" t="s">
-        <v>64</v>
-      </c>
-      <c r="M8" t="s">
-        <v>53</v>
-      </c>
-      <c r="N8" t="s">
-        <v>68</v>
-      </c>
-      <c r="O8" t="s">
-        <v>72</v>
-      </c>
-      <c r="P8" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>81</v>
-      </c>
-      <c r="R8" t="s">
-        <v>87</v>
-      </c>
-      <c r="S8" t="s">
-        <v>89</v>
-      </c>
-      <c r="T8" t="s">
-        <v>90</v>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F17" t="s">
+        <v>103</v>
+      </c>
+      <c r="G17" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" t="s">
+        <v>107</v>
+      </c>
+      <c r="I17" t="s">
+        <v>112</v>
+      </c>
+      <c r="J17" t="s">
+        <v>113</v>
+      </c>
+      <c r="K17" t="s">
+        <v>115</v>
+      </c>
+      <c r="L17" t="s">
+        <v>109</v>
+      </c>
+      <c r="M17" t="s">
+        <v>108</v>
+      </c>
+      <c r="N17" t="s">
+        <v>120</v>
+      </c>
+      <c r="O17" t="s">
+        <v>123</v>
+      </c>
+      <c r="P17" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update case data with new image upload analysis results
Added analysis for new document upload (images (2).jpg), updated case
registry JSON, refreshed decision reports and regenerated PDF reports.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/case_priority_system/case_results.xlsx
+++ b/case_priority_system/case_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="157">
   <si>
     <t>Case_File</t>
   </si>
@@ -115,13 +115,16 @@
     <t>Sample_FIR_Case_Report_Sexual_Assault.pdf</t>
   </si>
   <si>
+    <t>State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>_test_judgment.pdf</t>
+  </si>
+  <si>
     <t>Sample_Medium_Priority_FIR.pdf</t>
   </si>
   <si>
-    <t>State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800.PDF</t>
-  </si>
-  <si>
-    <t>_test_judgment.pdf</t>
+    <t>images (2).jpg</t>
   </si>
   <si>
     <t>Cipla Limited vs Union Of India</t>
@@ -163,15 +166,18 @@
     <t>Complainant, Victim, Accused</t>
   </si>
   <si>
-    <t>Mr. Arun Kumar, Unknown</t>
-  </si>
-  <si>
     <t>State of Karnataka, Union of India, Mysore Government Soap Factory, Mysore Sales International, Zonal Agents</t>
   </si>
   <si>
     <t>Sanjay Kumar, S/O Naresh Prasad, The State of Bihar through Principal Secretary Department of Excise and Prohibition, Government of Bihar, Patna, The District Magistrate Cum Collector, Nawada, The Senior Superintendent of Police, Nawada, The Superintendent of Police, Excise and Prohibition, Nawada, The Office in Charge, Kauakol Police Station, Nawada</t>
   </si>
   <si>
+    <t>Sample Medium Priority FIR</t>
+  </si>
+  <si>
+    <t>images (2)</t>
+  </si>
+  <si>
     <t>The parties, Cipla Limited vs Union Of India, are involved in a legal dispute. The document indicates central excise, excise duty, collector of central excise, classification list, elt. This case is classified as Excise/Tax because the record matches central excise, excise duty, collector of central excise, classification list, elt. Under the Constitution of India, the primary rights engaged are Article 265, Article 14, Article 19(1)(g).</t>
   </si>
   <si>
@@ -211,13 +217,16 @@
     <t>The complainant reports that the victim, a female aged [Age], was subjected to a sexual assault without her consent. The incident occurred at [Location] on [Date &amp; Time]. The victim informed a trusted individual and the matter was brought before the police. The complainant requests the investigation of the allegations, appropriate medical care, and legal action against the accused if the allegations are substantiated. This case falls under the Criminal/Violent category as it involves a serious assault on a vulnerable female victim.</t>
   </si>
   <si>
-    <t>Mr. Arun Kumar reported that his backpack, laptop, and accessories were stolen from a parked motorcycle. The theft occurred in the Market Road Parking Area. The case involves property damage and loss, as no physical injuries were reported. The investigation is ongoing, and the complainant seeks compensation for the loss. This case falls under General Civil as it deals with a property-related dispute and does not involve any immediate threat to life or ongoing violent incident.</t>
-  </si>
-  <si>
     <t>The State of Karnataka petitioned against the Union of India and the Mysore Government Soap Factory over excise duty and tax issues. The factory manufactures soap and sells it through a sole agent and zonal agents. The dispute centers around the trade discount allowed on the wholesale price of the soap. The State of Karnataka seeks to have the wholesale cash price of the soap determined without the 6% trade discount, arguing that the discount should only apply to the sales made to the retail dealers and approved buyers at the factory premises. The case involves constitutional issues related to the right to profession and the right to move the Supreme Court for enforcement of fundamental rights (Article 226).</t>
   </si>
   <si>
     <t>The case involves a writ petition seeking the release of a motorcycle seized by the police under the Bihar Prohibition and Excise Act. The petitioner, Sanjay Kumar, seeks the release of his motorcycle, which was seized in connection with a case registered under Section 30(a) of the Act. The case falls under the Excise/Tax category as it deals with the confiscation of property under the Bihar Prohibition and Excise Act, engaging Article 14 for the power imbalance and Article 21 for the protection of life and personal liberty.</t>
+  </si>
+  <si>
+    <t>The parties, Sample Medium Priority FIR, are involved in a legal dispute. The document indicates property, charge. This case is classified as Property/Land because the record matches property, charge. Under the Constitution of India, the primary rights engaged are Article 300A, Article 14, Article 21.</t>
+  </si>
+  <si>
+    <t>The parties, images (2), are involved in a legal dispute. The document indicates the facts of the dispute. This case is classified as General Civil because the record matches the facts of the dispute. Under the Constitution of India, the primary rights engaged are Article 14, Article 21.</t>
   </si>
   <si>
     <t>## STATE'S CONSTITUTIONAL ASSESSMENT
@@ -930,60 +939,6 @@
 (Neutral, Unbiased Analysis from the Perspective of the Judiciary)
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
-**Parties:** Mr. Arun Kumar, Unknown
-**Legal Category:** Excise/Tax
-**Brief Description:** Mr. Arun Kumar reported that his backpack, laptop, and accessories were stolen from a parked motorcycle. The theft occurred in the Market Road Parking Area. The case involves property damage and loss, as no physical injuries were reported. The investigation is ongoing, and the complainant seeks compensation for the loss. This case falls under General Civil as it deals with a property-related dispute and does not involve any immediate threat to life or ongoing violent incident.
-**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
-### II. CONSTITUTIONAL RIGHTS ENGAGED
-The following constitutional provisions are relevant to this matter:
-- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
-  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
-- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
-  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
-- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
-  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
-- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
-  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
-- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
-  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
-- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
-  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
-### III. SEVERITY &amp; URGENCY ASSESSMENT
-**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
-**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
-**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
-### IV. STATE'S DUTY UNDER THE CONSTITUTION
-Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
-### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
-**Vulnerability Level:** Low
-This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
-**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
-**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
-**Influence Level:** High
-Government bodies, large corporations, regulatory authorities, or politically powerful individuals
-**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
-**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
-### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
-- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
-  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
-- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
-  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
-- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
-  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
-- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
-  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
-### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
-**Assigned Priority:** Medium
-**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
-### VIII. FINAL OBSERVATION
-From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
-The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
-  </si>
-  <si>
-    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
-(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
-This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
-### I. SUBJECT MATTER
 **Parties:** State of Karnataka, Union of India, Mysore Government Soap Factory, Mysore Sales International, Zonal Agents
 **Legal Category:** Excise/Tax
 **Brief Description:** The State of Karnataka petitioned against the Union of India and the Mysore Government Soap Factory over excise duty and tax issues. The factory manufactures soap and sells it through a sole agent and zonal agents. The dispute centers around the trade discount allowed on the wholesale price of the soap. The State of Karnataka seeks to have the wholesale cash price of the soap determined without the 6% trade discount, arguing that the discount should only apply to the sales made to the retail dealers and approved buyers at the factory premises. The case involves constitutional issues related to the right to profession and the right to move the Supreme Court for enforcement of fundamental rights (Article 226).
@@ -1086,6 +1041,122 @@
 The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
   </si>
   <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Sample Medium Priority FIR
+**Legal Category:** Property/Land
+**Brief Description:** The parties, Sample Medium Priority FIR, are involved in a legal dispute. The document indicates property, charge. This case is classified as Property/Land because the record matches property, charge. Under the Constitution of India, the primary rights engaged are Article 300A, Article 14, Article 21.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 39 — Certain Principles of Policy to be Followed by the State**: The State shall direct its policy towards securing equal rights to an adequate means of livelihood, and that the ownership and control of material resources are so distributed as best to subserve the common good.
+  - Key principles: Adequate means of livelihood, Distribution of material resources for common good, Prevention of concentration of wealth, Protection of workers, children and women
+- ****[SECONDARY]** Article 46 — Promotion of Educational and Economic Interests of Weaker Sections**: The State shall promote with special care the educational and economic interests of the weaker sections of the people, and in particular of the Scheduled Castes and Scheduled Tribes, and shall protect them from social injustice and all forms of exploitation.
+  - Key principles: Special care for weaker sections, Protection of SC/ST from social injustice and exploitation
+- ****[SECONDARY]** Article 243G — Powers and Responsibilities of Panchayats**: The State legislature may endow Panchayats with such powers and authority as may be necessary to enable them to function as institutions of self-government, including in matters of land, water, agriculture and rural development.
+  - Key principles: Local self-government, Panchayat powers over land, water, agriculture
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 300A, no person shall be deprived of property except by authority of law. The State must ensure that land acquisition, eviction, and possession proceedings follow due process. When land disputes involve the homeless, tenants, or agricultural labourers, the right to livelihood under Article 21 is also engaged, requiring heightened judicial protection.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Doctrine of Legitimate Expectation**: A person who has a legitimate expectation based on a promise, practice or policy of the State is entitled to procedural fairness before that expectation is defeated.
+  - Application to this case: Applicable where administrative decisions frustrate settled practices, licences, or policies.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Property and land disputes primarily affect economic and possessory rights. However, when they involve the right to shelter or livelihood (Article 21), priority should be elevated. Routine property disputes without violence or immediate displacement risk warrant standard queue processing.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** images (2)
+**Legal Category:** Constitutional/Writ
+**Brief Description:** The parties, images (2), are involved in a legal dispute. The document indicates the facts of the dispute. This case is classified as General Civil because the record matches the facts of the dispute. Under the Constitution of India, the primary rights engaged are Article 14, Article 21.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = Low
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 32 — Remedies for Enforcement of Fundamental Rights**: The right to move the Supreme Court for the enforcement of fundamental rights is guaranteed.
+  - Key principles: Right to constitutional remedies, Writ jurisdiction of Supreme Court, Enforcement of fundamental rights
+- ****[PRIMARY]** Article 226 — Power of High Courts to Issue Certain Writs**: Every High Court shall have power to issue directions, orders, or writs for enforcement of fundamental rights and for any other purpose.
+  - Key principles: Writ jurisdiction of High Courts, Judicial review of state action, Enforcement of legal rights
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 227 — Power of Superintendence of High Courts**: Every High Court shall have superintendence over all courts and tribunals within its jurisdiction, and may call for returns, make rules, and settle forms to secure the proper administration of justice.
+  - Key principles: Superintendence over subordinate courts and tribunals, Administration of justice
+- ****[SECONDARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[SECONDARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** Low
+Individuals, small businesses, or parties of comparable standing
+**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
+**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Basic Structure**: The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.
+  - Application to this case: Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Colourable Legislation**: If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.
+  - Application to this case: Applicable where a statute purports to do one thing but in substance does another outside legislative competence.
+- **Doctrine of Harmonious Construction**: Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.
+  - Application to this case: Used when Articles or statutory provisions appear to overlap or clash.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Low
+**Category Rationale:** Constitutional writ matters directly engage fundamental rights and the rule of law. Cases involving imminent threats to life or liberty (habeas corpus) warrant the highest priority. Cases challenging administrative or quasi-judicial orders should receive priority proportionate to the gravity of the rights violation alleged and the urgency of the relief sought.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Low Priority**. 
+No urgent constitutional concern is identified. The matter should proceed in regular course. The court remains obligated under Article 14 to ensure that this matter is adjudicated fairly and without inordinate delay, even if it does not warrant special expedition.</t>
+  </si>
+  <si>
     <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
 **RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
 **RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
@@ -1110,6 +1181,17 @@
 **FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **High**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
   </si>
   <si>
+    <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**RULE 4 — Property/Land Dispute → Article 300A &amp; Livelihood:** Article 300A protects property rights. If livelihood (Article 21) is affected, priority should be elevated accordingly.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+  </si>
+  <si>
+    <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 4 — Constitutional/Writ Matter → Article 32/226 Jurisdiction:** The court's constitutional writ jurisdiction is engaged. Priority depends on the nature of the right sought to be enforced.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Low**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+  </si>
+  <si>
     <t>case_priority_system/decision_graphs\upload_test_decision_report.md</t>
   </si>
   <si>
@@ -1149,13 +1231,16 @@
     <t>case_priority_system/decision_graphs\Sample_FIR_Case_Report_Sexual_Assault_decision_report.md</t>
   </si>
   <si>
+    <t>case_priority_system/decision_graphs\State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\test_judgment_decision_report.md</t>
+  </si>
+  <si>
     <t>case_priority_system/decision_graphs\Sample_Medium_Priority_FIR_decision_report.md</t>
   </si>
   <si>
-    <t>case_priority_system/decision_graphs\State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800_decision_report.md</t>
-  </si>
-  <si>
-    <t>case_priority_system/decision_graphs\test_judgment_decision_report.md</t>
+    <t>case_priority_system/decision_graphs\images_2_decision_report.md</t>
   </si>
   <si>
     <t>Node 0: Severity is one of: Fatal, Major; case value = No Injury; result = No -&gt; Node 4: Influence / power imbalance is one of: High; case value = High; result = Yes -&gt; Leaf node 5 =&gt; Predicted Priority = Medium</t>
@@ -1185,12 +1270,21 @@
     <t>Customs/Import-Export</t>
   </si>
   <si>
+    <t>Property/Land</t>
+  </si>
+  <si>
+    <t>Constitutional/Writ</t>
+  </si>
+  <si>
     <t>Non-Violent</t>
   </si>
   <si>
     <t>Violent</t>
   </si>
   <si>
+    <t>Property</t>
+  </si>
+  <si>
     <t>No Injury</t>
   </si>
   <si>
@@ -1209,6 +1303,12 @@
     <t>Article 14 (Primary), Article 19(1)(g) (Primary), Article 300A (Primary), Article 265 (Secondary), Article 301 (Secondary), Article 21 (Secondary)</t>
   </si>
   <si>
+    <t>[{'article': 'Article 300A', 'title': 'Right to Property', 'primary': True}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True}, {'article': 'Article 39', 'title': 'Certain Principles of Policy to be Followed by the State', 'primary': False}, {'article': 'Article 46', 'title': 'Promotion of Educational and Economic Interests of Weaker Sections', 'primary': False}, {'article': 'Article 243G', 'title': 'Powers and Responsibilities of Panchayats', 'primary': False}]</t>
+  </si>
+  <si>
+    <t>[{'article': 'Article 32', 'title': 'Remedies for Enforcement of Fundamental Rights', 'primary': True}, {'article': 'Article 226', 'title': 'Power of High Courts to Issue Certain Writs', 'primary': True}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True}, {'article': 'Article 227', 'title': 'Power of Superintendence of High Courts', 'primary': False}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': False}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': False}, {'article': 'Article 51A', 'title': 'Fundamental Duties', 'primary': False}]</t>
+  </si>
+  <si>
     <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
   </si>
   <si>
@@ -1218,6 +1318,12 @@
     <t>The State must ensure that customs and import-export regulations are enforced lawfully and proportionately. Seizures, confiscations, and penalties must have legal sanction and must not arbitrarily deprive a person of their right to trade (Article 19(1)(g)) or property (Article 300A). The Directorate of Revenue Intelligence and customs authorities must act within the bounds of the law.</t>
   </si>
   <si>
+    <t>Under Article 300A, no person shall be deprived of property except by authority of law. The State must ensure that land acquisition, eviction, and possession proceedings follow due process. When land disputes involve the homeless, tenants, or agricultural labourers, the right to livelihood under Article 21 is also engaged, requiring heightened judicial protection.</t>
+  </si>
+  <si>
+    <t>The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.</t>
+  </si>
+  <si>
     <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Reasonable Classification', 'description': 'Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.', 'application': 'Used to test whether differential treatment of litigants or groups is constitutional.'}]</t>
   </si>
   <si>
@@ -1228,6 +1334,12 @@
   </si>
   <si>
     <t>Doctrine of Proportionality; Principle of Natural Justice — Audi Alteram Partem; Doctrine of Legitimate Expectation</t>
+  </si>
+  <si>
+    <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Doctrine of Legitimate Expectation', 'description': 'A person who has a legitimate expectation based on a promise, practice or policy of the State is entitled to procedural fairness before that expectation is defeated.', 'application': 'Applicable where administrative decisions frustrate settled practices, licences, or policies.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}]</t>
+  </si>
+  <si>
+    <t>[{'name': 'Doctrine of Basic Structure', 'description': 'The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.', 'application': 'Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.'}, {'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Colourable Legislation', 'description': 'If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.', 'application': 'Applicable where a statute purports to do one thing but in substance does another outside legislative competence.'}, {'name': 'Doctrine of Harmonious Construction', 'description': 'Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.', 'application': 'Used when Articles or statutory provisions appear to overlap or clash.'}]</t>
   </si>
   <si>
     <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
@@ -1257,7 +1369,31 @@
 **Category-Specific Analysis — Customs/Import-Export:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
   </si>
   <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Property/Land:** Property rights under Article 300A are constitutional but not absolute. The priority should consider whether the dispute involves livelihood (Article 21) or mere property entitlement.</t>
+  </si>
+  <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Category-Specific Analysis — Constitutional/Writ:** Writ matters directly engage the court's constitutional jurisdiction under Articles 32 and 226. The priority should reflect the nature of the right sought to be enforced — habeas corpus (life/liberty) cases require the highest priority.</t>
+  </si>
+  <si>
     <t>case_priority_system\reports\_upload_test_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\Sample_Medium_Priority_FIR_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\images (2)_report.pdf</t>
+  </si>
+  <si>
+    <t>ANV-2026-0004</t>
+  </si>
+  <si>
+    <t>FIR</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -1615,7 +1751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1685,55 +1821,55 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="G2" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H2" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J2" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L2" t="s">
+        <v>116</v>
+      </c>
+      <c r="M2" t="s">
         <v>115</v>
       </c>
-      <c r="L2" t="s">
-        <v>109</v>
-      </c>
-      <c r="M2" t="s">
-        <v>108</v>
-      </c>
       <c r="N2" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="O2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P2" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="Q2" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="R2" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1741,52 +1877,52 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="G3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="H3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="I3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="J3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="K3" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="L3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="M3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="N3" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="O3" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="P3" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="Q3" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1794,52 +1930,52 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J4" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K4" t="s">
+        <v>125</v>
+      </c>
+      <c r="L4" t="s">
+        <v>116</v>
+      </c>
+      <c r="M4" t="s">
         <v>115</v>
       </c>
-      <c r="L4" t="s">
-        <v>109</v>
-      </c>
-      <c r="M4" t="s">
-        <v>108</v>
-      </c>
       <c r="N4" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O4" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P4" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q4" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1847,52 +1983,52 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H5" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I5" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J5" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K5" t="s">
+        <v>125</v>
+      </c>
+      <c r="L5" t="s">
+        <v>116</v>
+      </c>
+      <c r="M5" t="s">
         <v>115</v>
       </c>
-      <c r="L5" t="s">
-        <v>109</v>
-      </c>
-      <c r="M5" t="s">
-        <v>108</v>
-      </c>
       <c r="N5" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O5" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P5" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q5" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1900,52 +2036,52 @@
         <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G6" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H6" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I6" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J6" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K6" t="s">
+        <v>125</v>
+      </c>
+      <c r="L6" t="s">
+        <v>116</v>
+      </c>
+      <c r="M6" t="s">
         <v>115</v>
       </c>
-      <c r="L6" t="s">
-        <v>109</v>
-      </c>
-      <c r="M6" t="s">
-        <v>108</v>
-      </c>
       <c r="N6" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O6" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P6" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q6" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1953,52 +2089,52 @@
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E7" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F7" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="H7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="I7" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J7" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K7" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="L7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="M7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="N7" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O7" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P7" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q7" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -2006,52 +2142,52 @@
         <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E8" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G8" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H8" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I8" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J8" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K8" t="s">
+        <v>125</v>
+      </c>
+      <c r="L8" t="s">
+        <v>116</v>
+      </c>
+      <c r="M8" t="s">
         <v>115</v>
       </c>
-      <c r="L8" t="s">
-        <v>109</v>
-      </c>
-      <c r="M8" t="s">
-        <v>108</v>
-      </c>
       <c r="N8" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O8" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P8" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q8" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -2059,52 +2195,52 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E9" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F9" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G9" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H9" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I9" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J9" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K9" t="s">
+        <v>125</v>
+      </c>
+      <c r="L9" t="s">
+        <v>116</v>
+      </c>
+      <c r="M9" t="s">
         <v>115</v>
       </c>
-      <c r="L9" t="s">
-        <v>109</v>
-      </c>
-      <c r="M9" t="s">
-        <v>108</v>
-      </c>
       <c r="N9" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O9" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P9" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q9" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -2112,52 +2248,52 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F10" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G10" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I10" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J10" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K10" t="s">
+        <v>125</v>
+      </c>
+      <c r="L10" t="s">
+        <v>116</v>
+      </c>
+      <c r="M10" t="s">
         <v>115</v>
       </c>
-      <c r="L10" t="s">
-        <v>109</v>
-      </c>
-      <c r="M10" t="s">
-        <v>108</v>
-      </c>
       <c r="N10" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O10" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P10" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q10" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -2165,52 +2301,52 @@
         <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E11" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="G11" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="H11" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="I11" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="J11" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="K11" t="s">
+        <v>126</v>
+      </c>
+      <c r="L11" t="s">
+        <v>115</v>
+      </c>
+      <c r="M11" t="s">
         <v>116</v>
       </c>
-      <c r="L11" t="s">
-        <v>108</v>
-      </c>
-      <c r="M11" t="s">
-        <v>109</v>
-      </c>
       <c r="N11" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="O11" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="P11" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="Q11" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -2218,52 +2354,52 @@
         <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F12" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="G12" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H12" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I12" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="J12" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K12" t="s">
+        <v>125</v>
+      </c>
+      <c r="L12" t="s">
+        <v>116</v>
+      </c>
+      <c r="M12" t="s">
         <v>115</v>
       </c>
-      <c r="L12" t="s">
-        <v>109</v>
-      </c>
-      <c r="M12" t="s">
-        <v>108</v>
-      </c>
       <c r="N12" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="O12" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="P12" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="Q12" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -2271,52 +2407,52 @@
         <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G13" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I13" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J13" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K13" t="s">
+        <v>125</v>
+      </c>
+      <c r="L13" t="s">
+        <v>116</v>
+      </c>
+      <c r="M13" t="s">
         <v>115</v>
       </c>
-      <c r="L13" t="s">
-        <v>109</v>
-      </c>
-      <c r="M13" t="s">
-        <v>108</v>
-      </c>
       <c r="N13" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O13" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P13" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q13" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -2324,52 +2460,52 @@
         <v>32</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F14" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G14" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="H14" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="I14" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="J14" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="K14" t="s">
+        <v>126</v>
+      </c>
+      <c r="L14" t="s">
+        <v>115</v>
+      </c>
+      <c r="M14" t="s">
         <v>116</v>
       </c>
-      <c r="L14" t="s">
-        <v>108</v>
-      </c>
-      <c r="M14" t="s">
-        <v>109</v>
-      </c>
       <c r="N14" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="O14" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="P14" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="Q14" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -2377,52 +2513,52 @@
         <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F15" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G15" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H15" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I15" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J15" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K15" t="s">
+        <v>125</v>
+      </c>
+      <c r="L15" t="s">
+        <v>116</v>
+      </c>
+      <c r="M15" t="s">
         <v>115</v>
       </c>
-      <c r="L15" t="s">
-        <v>109</v>
-      </c>
-      <c r="M15" t="s">
-        <v>108</v>
-      </c>
       <c r="N15" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O15" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P15" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="Q15" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -2430,105 +2566,176 @@
         <v>34</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F16" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="G16" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H16" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I16" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="J16" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="K16" t="s">
+        <v>125</v>
+      </c>
+      <c r="L16" t="s">
+        <v>116</v>
+      </c>
+      <c r="M16" t="s">
         <v>115</v>
       </c>
-      <c r="L16" t="s">
-        <v>109</v>
-      </c>
-      <c r="M16" t="s">
-        <v>108</v>
-      </c>
       <c r="N16" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="O16" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="P16" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="Q16" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:20">
       <c r="A17" t="s">
         <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G17" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H17" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I17" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="J17" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="K17" t="s">
+        <v>125</v>
+      </c>
+      <c r="L17" t="s">
+        <v>116</v>
+      </c>
+      <c r="M17" t="s">
         <v>115</v>
       </c>
-      <c r="L17" t="s">
-        <v>109</v>
-      </c>
-      <c r="M17" t="s">
-        <v>108</v>
-      </c>
       <c r="N17" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="O17" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="P17" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="Q17" t="s">
+        <v>149</v>
+      </c>
+      <c r="R17" t="s">
+        <v>152</v>
+      </c>
+      <c r="S17" t="s">
+        <v>154</v>
+      </c>
+      <c r="T17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" t="s">
+        <v>93</v>
+      </c>
+      <c r="F18" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" t="s">
+        <v>110</v>
+      </c>
+      <c r="H18" t="s">
+        <v>116</v>
+      </c>
+      <c r="I18" t="s">
+        <v>121</v>
+      </c>
+      <c r="J18" t="s">
+        <v>122</v>
+      </c>
+      <c r="K18" t="s">
+        <v>125</v>
+      </c>
+      <c r="L18" t="s">
+        <v>116</v>
+      </c>
+      <c r="M18" t="s">
+        <v>116</v>
+      </c>
+      <c r="N18" t="s">
         <v>132</v>
+      </c>
+      <c r="O18" t="s">
+        <v>137</v>
+      </c>
+      <c r="P18" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>150</v>
+      </c>
+      <c r="R18" t="s">
+        <v>153</v>
+      </c>
+      <c r="S18" t="s">
+        <v>154</v>
+      </c>
+      <c r="T18" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update case data and reports with latest analysis results
Refresh Excel case results, decision path reports, and generated
PDFs to reflect the latest pipeline run output.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/case_priority_system/case_results.xlsx
+++ b/case_priority_system/case_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="163">
   <si>
     <t>Case_File</t>
   </si>
@@ -103,30 +103,30 @@
     <t>Deepak_Extrusion_And_Anr_vs_J_T_Chopra_Assistant_Collector_Of_on_1_January_1800.PDF</t>
   </si>
   <si>
+    <t>Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>Rakhra_Sports_Private_Ltd_And_Others_vs_Khraitilal_Rakhra_And_Others_on_1_January_1800.PDF</t>
+  </si>
+  <si>
+    <t>Sample_FIR_Case_Report_Sexual_Assault.pdf</t>
+  </si>
+  <si>
+    <t>_test_judgment.pdf</t>
+  </si>
+  <si>
+    <t>Sample_Medium_Priority_FIR.pdf</t>
+  </si>
+  <si>
+    <t>images (2).jpg</t>
+  </si>
+  <si>
     <t>Fictional_Case_Report_Test.pdf</t>
   </si>
   <si>
-    <t>Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800.PDF</t>
-  </si>
-  <si>
-    <t>Rakhra_Sports_Private_Ltd_And_Others_vs_Khraitilal_Rakhra_And_Others_on_1_January_1800.PDF</t>
-  </si>
-  <si>
-    <t>Sample_FIR_Case_Report_Sexual_Assault.pdf</t>
-  </si>
-  <si>
     <t>State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800.PDF</t>
   </si>
   <si>
-    <t>_test_judgment.pdf</t>
-  </si>
-  <si>
-    <t>Sample_Medium_Priority_FIR.pdf</t>
-  </si>
-  <si>
-    <t>images (2).jpg</t>
-  </si>
-  <si>
     <t>Cipla Limited vs Union Of India</t>
   </si>
   <si>
@@ -154,28 +154,28 @@
     <t>Deepak Extrusion And Anr., J.T. Chopra Assistant Collector Of ...</t>
   </si>
   <si>
+    <t>Pooja Exporters, Assistant Director, D.R.I.</t>
+  </si>
+  <si>
+    <t>Rakhra Sports Private Ltd. And Others, Khraitilal Rakhra And Others</t>
+  </si>
+  <si>
+    <t>Complainant, Victim, Accused</t>
+  </si>
+  <si>
+    <t>Sanjay Kumar, S/O Naresh Prasad, The State of Bihar through Principal Secretary Department of Excise and Prohibition, Government of Bihar, Patna, The District Magistrate Cum Collector, Nawada, The Senior Superintendent of Police, Nawada, The Superintendent of Police, Excise and Prohibition, Nawada, The Office in Charge, Kauakol Police Station, Nawada</t>
+  </si>
+  <si>
+    <t>Sample Medium Priority FIR</t>
+  </si>
+  <si>
+    <t>images (2)</t>
+  </si>
+  <si>
     <t>Emma Carter, Two Unidentified Males</t>
   </si>
   <si>
-    <t>Pooja Exporters, Assistant Director, D.R.I.</t>
-  </si>
-  <si>
-    <t>Rakhra Sports Private Ltd. And Others, Khraitilal Rakhra And Others</t>
-  </si>
-  <si>
-    <t>Complainant, Victim, Accused</t>
-  </si>
-  <si>
-    <t>State of Karnataka, Union of India, Mysore Government Soap Factory, Mysore Sales International, Zonal Agents</t>
-  </si>
-  <si>
-    <t>Sanjay Kumar, S/O Naresh Prasad, The State of Bihar through Principal Secretary Department of Excise and Prohibition, Government of Bihar, Patna, The District Magistrate Cum Collector, Nawada, The Senior Superintendent of Police, Nawada, The Superintendent of Police, Excise and Prohibition, Nawada, The Office in Charge, Kauakol Police Station, Nawada</t>
-  </si>
-  <si>
-    <t>Sample Medium Priority FIR</t>
-  </si>
-  <si>
-    <t>images (2)</t>
+    <t>State of Karnataka, Union of India, U.L.Narayana Rao, Respondents</t>
   </si>
   <si>
     <t>The parties, Cipla Limited vs Union Of India, are involved in a legal dispute. The document indicates central excise, excise duty, collector of central excise, classification list, elt. This case is classified as Excise/Tax because the record matches central excise, excise duty, collector of central excise, classification list, elt. Under the Constitution of India, the primary rights engaged are Article 265, Article 14, Article 19(1)(g).</t>
@@ -205,9 +205,6 @@
     <t>The petitioners, Deepak Extrusion And Anr., challenge the constitutional validity of the amendment to Section 2(f) and Tariff Item 27 of the Central Excise Act. The case involves the levy of excise duty on aluminium containers that have been lacquered or printed. The Department argues that lacquering and printing are also a form of manufacture, while the petitioners contend that these processes are ancillary to the manufacture of the final product. The case raises questions about the scope of the term 'manufacture' in the Excise Act and the applicability of the decision in Empire Industries Ltd. v. Union of India to aluminium products.</t>
   </si>
   <si>
-    <t>Emma Carter, a store manager, was seriously injured during an armed robbery at a convenience store. Two unidentified males, one armed with a handgun and the other with a metal crowbar, assaulted her and stole cash and merchandise. The victim was hospitalized in ICU. The case involves serious physical harm and the potential for permanent disability, engaging Article 21 of the Constitution of India.</t>
-  </si>
-  <si>
     <t>Pooja Exporters, a registered partnership firm, sought a writ of mandamus and prohibition against the Assistant Director, D.R.I. to release 51 bales of 100% mulberry raw silk seized by customs authorities. The petitioner argued that the seizure was illegal and in violation of their import licence, while the respondents contended that the petitioner had violated the actual user condition of the licence. The case falls under the Customs/Import-Export category as it involves customs seizure and import licence issues.</t>
   </si>
   <si>
@@ -217,9 +214,6 @@
     <t>The complainant reports that the victim, a female aged [Age], was subjected to a sexual assault without her consent. The incident occurred at [Location] on [Date &amp; Time]. The victim informed a trusted individual and the matter was brought before the police. The complainant requests the investigation of the allegations, appropriate medical care, and legal action against the accused if the allegations are substantiated. This case falls under the Criminal/Violent category as it involves a serious assault on a vulnerable female victim.</t>
   </si>
   <si>
-    <t>The State of Karnataka petitioned against the Union of India and the Mysore Government Soap Factory over excise duty and tax issues. The factory manufactures soap and sells it through a sole agent and zonal agents. The dispute centers around the trade discount allowed on the wholesale price of the soap. The State of Karnataka seeks to have the wholesale cash price of the soap determined without the 6% trade discount, arguing that the discount should only apply to the sales made to the retail dealers and approved buyers at the factory premises. The case involves constitutional issues related to the right to profession and the right to move the Supreme Court for enforcement of fundamental rights (Article 226).</t>
-  </si>
-  <si>
     <t>The case involves a writ petition seeking the release of a motorcycle seized by the police under the Bihar Prohibition and Excise Act. The petitioner, Sanjay Kumar, seeks the release of his motorcycle, which was seized in connection with a case registered under Section 30(a) of the Act. The case falls under the Excise/Tax category as it deals with the confiscation of property under the Bihar Prohibition and Excise Act, engaging Article 14 for the power imbalance and Article 21 for the protection of life and personal liberty.</t>
   </si>
   <si>
@@ -227,6 +221,12 @@
   </si>
   <si>
     <t>The parties, images (2), are involved in a legal dispute. The document indicates the facts of the dispute. This case is classified as General Civil because the record matches the facts of the dispute. Under the Constitution of India, the primary rights engaged are Article 14, Article 21.</t>
+  </si>
+  <si>
+    <t>Emma Carter, a store manager, was assaulted with a crowbar and handgun during an armed robbery at a convenience store. She sustained severe head injuries and was hospitalized. The two suspects fled the scene, leaving the victim vulnerable and in need of urgent legal intervention. This case falls under the Criminal/Violent category as it involves a violent assault and the potential for serious injury, engaging Article 21 of the Constitution for the protection of life and personal liberty.</t>
+  </si>
+  <si>
+    <t>This case involves a dispute between the State of Karnataka and the Union of India regarding the excise duty on soap manufactured by the petitioner. The petitioner seeks to determine the percentage of trade discount allowable under the Excise Act, while the Union of India argues that the wholesale market for the soap does not exist. The petitioner claims that the agreements with the sole selling agent and zonal agents should be the basis for determining the price of the soap, and not isolated sales. The case falls under the Excise/Tax category as it deals with excise duty on soap manufactured by the petitioner.</t>
   </si>
   <si>
     <t>## STATE'S CONSTITUTIONAL ASSESSMENT
@@ -721,62 +721,6 @@
 (Neutral, Unbiased Analysis from the Perspective of the Judiciary)
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
-**Parties:** Emma Carter, Two Unidentified Males
-**Legal Category:** Criminal/Violent
-**Brief Description:** Emma Carter, a store manager, was seriously injured during an armed robbery at a convenience store. Two unidentified males, one armed with a handgun and the other with a metal crowbar, assaulted her and stole cash and merchandise. The victim was hospitalized in ICU. The case involves serious physical harm and the potential for permanent disability, engaging Article 21 of the Constitution of India.
-**Extracted Parameters:** Severity = Major, Vulnerability = High, Influence/ Power Imbalance = Low
-### II. CONSTITUTIONAL RIGHTS ENGAGED
-The following constitutional provisions are relevant to this matter:
-- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
-  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
-- ****[PRIMARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
-  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
-- ****[PRIMARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
-  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
-- ****[SECONDARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
-  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
-- ****[SECONDARY]** Article 17 — Abolition of Untouchability**: Untouchability is abolished and its practice in any form is forbidden. The enforcement of any disability arising out of untouchability shall be an offence punishable in accordance with law.
-  - Key principles: Abolition of untouchability, Enforcement of disabilities is an offence, Protection of SC/ST communities
-- ****[SECONDARY]** Article 23 — Prohibition of Traffic in Human Beings and Forced Labour**: Traffic in human beings and begar and other similar forms of forced labour are prohibited. Any contravention of this provision shall be an offence punishable in accordance with law.
-  - Key principles: Prohibition of human trafficking, Prohibition of forced labour and begar
-- ****[SECONDARY]** Article 24 — Prohibition of Employment of Children in Factories**: No child below the age of fourteen years shall be employed to work in any factory or mine or engaged in any other hazardous employment.
-  - Key principles: No child labour below 14 in hazardous work, Protection of children from exploitation
-- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
-  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
-### III. SEVERITY &amp; URGENCY ASSESSMENT
-**Primary Article:** Article 21
-**Analysis:** The right to life under Article 21 includes the right to live with dignity and the right to health. Major injuries — especially those requiring hospitalisation, causing permanent disability, or posing life-threatening complications — constitute a serious interference with personal liberty and bodily integrity. The State must ensure prompt access to medical care, investigation of the incident, and accountability. Each day of delay risks permanent aggravation of the harm.
-**Urgency Classification:** High — bodily integrity and dignity are seriously compromised.
-### IV. STATE'S DUTY UNDER THE CONSTITUTION
-The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.
-### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
-**Vulnerability Level:** High
-This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
-**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
-**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
-**Influence Level:** Low
-Individuals, small businesses, or parties of comparable standing
-**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
-**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
-### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
-- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
-  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
-- **Doctrine of Parens Patriae**: The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.
-  - Application to this case: Critical for cases involving vulnerable victims — the state must act as guardian.
-- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
-  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
-### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
-**Assigned Priority:** High
-**Category Rationale:** Cases involving violent crime directly implicate the most fundamental right under the Constitution — the right to life. The state's failure to accord such cases the highest priority would constitute a violation of its affirmative obligation under Article 21 to protect life and ensure access to justice.
-### VIII. FINAL OBSERVATION
-From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **High Priority**. 
-This is constitutionally appropriate and reflects the gravity of the rights engaged. The court is directed to list this matter expeditiously, ensuring that no procedural delay undermines the constitutional rights at stake. The State must accord this case the attention and resources commensurate with its priority level.</t>
-  </si>
-  <si>
-    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
-(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
-This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
-### I. SUBJECT MATTER
 **Parties:** Pooja Exporters, Assistant Director, D.R.I.
 **Legal Category:** Customs/Import-Export
 **Brief Description:** Pooja Exporters, a registered partnership firm, sought a writ of mandamus and prohibition against the Assistant Director, D.R.I. to release 51 bales of 100% mulberry raw silk seized by customs authorities. The petitioner argued that the seizure was illegal and in violation of their import licence, while the respondents contended that the petitioner had violated the actual user condition of the licence. The case falls under the Customs/Import-Export category as it involves customs seizure and import licence issues.
@@ -933,60 +877,6 @@
 ### VIII. FINAL OBSERVATION
 From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **High Priority**. 
 This is constitutionally appropriate and reflects the gravity of the rights engaged. The court is directed to list this matter expeditiously, ensuring that no procedural delay undermines the constitutional rights at stake. The State must accord this case the attention and resources commensurate with its priority level.</t>
-  </si>
-  <si>
-    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
-(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
-This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
-### I. SUBJECT MATTER
-**Parties:** State of Karnataka, Union of India, Mysore Government Soap Factory, Mysore Sales International, Zonal Agents
-**Legal Category:** Excise/Tax
-**Brief Description:** The State of Karnataka petitioned against the Union of India and the Mysore Government Soap Factory over excise duty and tax issues. The factory manufactures soap and sells it through a sole agent and zonal agents. The dispute centers around the trade discount allowed on the wholesale price of the soap. The State of Karnataka seeks to have the wholesale cash price of the soap determined without the 6% trade discount, arguing that the discount should only apply to the sales made to the retail dealers and approved buyers at the factory premises. The case involves constitutional issues related to the right to profession and the right to move the Supreme Court for enforcement of fundamental rights (Article 226).
-**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
-### II. CONSTITUTIONAL RIGHTS ENGAGED
-The following constitutional provisions are relevant to this matter:
-- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
-  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
-- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
-  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
-- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
-  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
-- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
-  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
-- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
-  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
-- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
-  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
-### III. SEVERITY &amp; URGENCY ASSESSMENT
-**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
-**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
-**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
-### IV. STATE'S DUTY UNDER THE CONSTITUTION
-Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
-### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
-**Vulnerability Level:** Low
-This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
-**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
-**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
-**Influence Level:** High
-Government bodies, large corporations, regulatory authorities, or politically powerful individuals
-**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
-**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
-### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
-- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
-  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
-- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
-  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
-- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
-  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
-- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
-  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
-### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
-**Assigned Priority:** Medium
-**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
-### VIII. FINAL OBSERVATION
-From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
-The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
   </si>
   <si>
     <t>## STATE'S CONSTITUTIONAL ASSESSMENT
@@ -1157,6 +1047,116 @@
 No urgent constitutional concern is identified. The matter should proceed in regular course. The court remains obligated under Article 14 to ensure that this matter is adjudicated fairly and without inordinate delay, even if it does not warrant special expedition.</t>
   </si>
   <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Emma Carter, Two Unidentified Males
+**Legal Category:** Criminal/Violent
+**Brief Description:** Emma Carter, a store manager, was assaulted with a crowbar and handgun during an armed robbery at a convenience store. She sustained severe head injuries and was hospitalized. The two suspects fled the scene, leaving the victim vulnerable and in need of urgent legal intervention. This case falls under the Criminal/Violent category as it involves a violent assault and the potential for serious injury, engaging Article 21 of the Constitution for the protection of life and personal liberty.
+**Extracted Parameters:** Severity = Major, Vulnerability = High, Influence/ Power Imbalance = Low
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[PRIMARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[PRIMARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[SECONDARY]** Article 17 — Abolition of Untouchability**: Untouchability is abolished and its practice in any form is forbidden. The enforcement of any disability arising out of untouchability shall be an offence punishable in accordance with law.
+  - Key principles: Abolition of untouchability, Enforcement of disabilities is an offence, Protection of SC/ST communities
+- ****[SECONDARY]** Article 23 — Prohibition of Traffic in Human Beings and Forced Labour**: Traffic in human beings and begar and other similar forms of forced labour are prohibited. Any contravention of this provision shall be an offence punishable in accordance with law.
+  - Key principles: Prohibition of human trafficking, Prohibition of forced labour and begar
+- ****[SECONDARY]** Article 24 — Prohibition of Employment of Children in Factories**: No child below the age of fourteen years shall be employed to work in any factory or mine or engaged in any other hazardous employment.
+  - Key principles: No child labour below 14 in hazardous work, Protection of children from exploitation
+- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
+  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 21
+**Analysis:** The right to life under Article 21 includes the right to live with dignity and the right to health. Major injuries — especially those requiring hospitalisation, causing permanent disability, or posing life-threatening complications — constitute a serious interference with personal liberty and bodily integrity. The State must ensure prompt access to medical care, investigation of the incident, and accountability. Each day of delay risks permanent aggravation of the harm.
+**Urgency Classification:** High — bodily integrity and dignity are seriously compromised.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** High
+This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
+**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
+**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
+**Influence Level:** Low
+Individuals, small businesses, or parties of comparable standing
+**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
+**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Doctrine of Parens Patriae**: The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.
+  - Application to this case: Critical for cases involving vulnerable victims — the state must act as guardian.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** High
+**Category Rationale:** Cases involving violent crime directly implicate the most fundamental right under the Constitution — the right to life. The state's failure to accord such cases the highest priority would constitute a violation of its affirmative obligation under Article 21 to protect life and ensure access to justice.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **High Priority**. 
+This is constitutionally appropriate and reflects the gravity of the rights engaged. The court is directed to list this matter expeditiously, ensuring that no procedural delay undermines the constitutional rights at stake. The State must accord this case the attention and resources commensurate with its priority level.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** State of Karnataka, Union of India, U.L.Narayana Rao, Respondents
+**Legal Category:** Excise/Tax
+**Brief Description:** This case involves a dispute between the State of Karnataka and the Union of India regarding the excise duty on soap manufactured by the petitioner. The petitioner seeks to determine the percentage of trade discount allowable under the Excise Act, while the Union of India argues that the wholesale market for the soap does not exist. The petitioner claims that the agreements with the sole selling agent and zonal agents should be the basis for determining the price of the soap, and not isolated sales. The case falls under the Excise/Tax category as it deals with excise duty on soap manufactured by the petitioner.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
     <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
 **RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
 **RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
@@ -1219,30 +1219,30 @@
     <t>case_priority_system/decision_graphs\Deepak_Extrusion_And_Anr_vs_J_T_Chopra_Assistant_Collector_Of_on_1_January_1800_decision_report.md</t>
   </si>
   <si>
+    <t>case_priority_system/decision_graphs\Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Rakhra_Sports_Private_Ltd_And_Others_vs_Khraitilal_Rakhra_And_Others_on_1_January_1800_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Sample_FIR_Case_Report_Sexual_Assault_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\test_judgment_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Sample_Medium_Priority_FIR_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\images_2_decision_report.md</t>
+  </si>
+  <si>
     <t>case_priority_system/decision_graphs\Fictional_Case_Report_Test_decision_report.md</t>
   </si>
   <si>
-    <t>case_priority_system/decision_graphs\Pooja_Exporters_vs_Assistant_Director_D_R_I_on_1_January_1800_decision_report.md</t>
-  </si>
-  <si>
-    <t>case_priority_system/decision_graphs\Rakhra_Sports_Private_Ltd_And_Others_vs_Khraitilal_Rakhra_And_Others_on_1_January_1800_decision_report.md</t>
-  </si>
-  <si>
-    <t>case_priority_system/decision_graphs\Sample_FIR_Case_Report_Sexual_Assault_decision_report.md</t>
-  </si>
-  <si>
     <t>case_priority_system/decision_graphs\State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800_decision_report.md</t>
   </si>
   <si>
-    <t>case_priority_system/decision_graphs\test_judgment_decision_report.md</t>
-  </si>
-  <si>
-    <t>case_priority_system/decision_graphs\Sample_Medium_Priority_FIR_decision_report.md</t>
-  </si>
-  <si>
-    <t>case_priority_system/decision_graphs\images_2_decision_report.md</t>
-  </si>
-  <si>
     <t>Node 0: Severity is one of: Fatal, Major; case value = No Injury; result = No -&gt; Node 4: Influence / power imbalance is one of: High; case value = High; result = Yes -&gt; Leaf node 5 =&gt; Predicted Priority = Medium</t>
   </si>
   <si>
@@ -1309,6 +1309,9 @@
     <t>[{'article': 'Article 32', 'title': 'Remedies for Enforcement of Fundamental Rights', 'primary': True}, {'article': 'Article 226', 'title': 'Power of High Courts to Issue Certain Writs', 'primary': True}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True}, {'article': 'Article 227', 'title': 'Power of Superintendence of High Courts', 'primary': False}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': False}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': False}, {'article': 'Article 51A', 'title': 'Fundamental Duties', 'primary': False}]</t>
   </si>
   <si>
+    <t>[{'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': True}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': True}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': False}, {'article': 'Article 17', 'title': 'Abolition of Untouchability', 'primary': False}, {'article': 'Article 23', 'title': 'Prohibition of Traffic in Human Beings and Forced Labour', 'primary': False}, {'article': 'Article 24', 'title': 'Prohibition of Employment of Children in Factories', 'primary': False}, {'article': 'Article 39A', 'title': 'Equal Justice and Free Legal Aid', 'primary': False}]</t>
+  </si>
+  <si>
     <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
   </si>
   <si>
@@ -1340,6 +1343,9 @@
   </si>
   <si>
     <t>[{'name': 'Doctrine of Basic Structure', 'description': 'The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.', 'application': 'Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.'}, {'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Colourable Legislation', 'description': 'If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.', 'application': 'Applicable where a statute purports to do one thing but in substance does another outside legislative competence.'}, {'name': 'Doctrine of Harmonious Construction', 'description': 'Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.', 'application': 'Used when Articles or statutory provisions appear to overlap or clash.'}]</t>
+  </si>
+  <si>
+    <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Doctrine of Parens Patriae', 'description': 'The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.', 'application': 'Critical for cases involving vulnerable victims — the state must act as guardian.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}]</t>
   </si>
   <si>
     <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
@@ -1358,6 +1364,11 @@
 **Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
   </si>
   <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Customs/Import-Export:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
+  </si>
+  <si>
     <t>**Primary Interest — Right to Life &amp; Bodily Integrity (Article 21):** The severity level 'Major' indicates that the right to life or physical integrity has been seriously compromised. Under Article 21, this is the weightiest constitutional interest and must take precedence over all other considerations. The state's duty to protect life is non-derogable and non-delegable.
 **Assessment:** The High priority correctly reflects the primacy of Article 21 rights. This is constitutionally appropriate and proportionate to the gravity of the harm.
 **Vulnerability Analysis — Special State Obligation:** A vulnerable party is involved. The Doctrine of Parens Patriae and Articles 15(3), 15(4), 39, and 39A impose a heightened duty on the state to protect the vulnerable. This factor strongly supports High priority to prevent further harm or injustice.
@@ -1366,11 +1377,6 @@
   <si>
     <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
 **Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
-**Category-Specific Analysis — Customs/Import-Export:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
-  </si>
-  <si>
-    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
-**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
 **Category-Specific Analysis — Property/Land:** Property rights under Article 300A are constitutional but not absolute. The priority should consider whether the dispute involves livelihood (Article 21) or mere property entitlement.</t>
   </si>
   <si>
@@ -1387,7 +1393,19 @@
     <t>case_priority_system\reports\images (2)_report.pdf</t>
   </si>
   <si>
+    <t>case_priority_system\reports\Fictional_Case_Report_Test_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\State_Of_Karnataka_vs_Union_Of_India_And_Ors_on_1_January_1800_report.pdf</t>
+  </si>
+  <si>
     <t>ANV-2026-0004</t>
+  </si>
+  <si>
+    <t>ANV-2026-0007</t>
+  </si>
+  <si>
+    <t>ANV-2026-0008</t>
   </si>
   <si>
     <t>FIR</t>
@@ -1860,16 +1878,16 @@
         <v>127</v>
       </c>
       <c r="O2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="R2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1916,13 +1934,13 @@
         <v>128</v>
       </c>
       <c r="O3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1969,13 +1987,13 @@
         <v>129</v>
       </c>
       <c r="O4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -2022,13 +2040,13 @@
         <v>129</v>
       </c>
       <c r="O5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -2075,13 +2093,13 @@
         <v>129</v>
       </c>
       <c r="O6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -2128,13 +2146,13 @@
         <v>129</v>
       </c>
       <c r="O7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -2181,13 +2199,13 @@
         <v>129</v>
       </c>
       <c r="O8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q8" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -2234,13 +2252,13 @@
         <v>129</v>
       </c>
       <c r="O9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -2287,13 +2305,13 @@
         <v>129</v>
       </c>
       <c r="O10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -2310,43 +2328,43 @@
         <v>80</v>
       </c>
       <c r="E11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F11" t="s">
         <v>103</v>
       </c>
       <c r="G11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H11" t="s">
+        <v>114</v>
+      </c>
+      <c r="I11" t="s">
+        <v>119</v>
+      </c>
+      <c r="J11" t="s">
+        <v>122</v>
+      </c>
+      <c r="K11" t="s">
+        <v>125</v>
+      </c>
+      <c r="L11" t="s">
+        <v>116</v>
+      </c>
+      <c r="M11" t="s">
         <v>115</v>
       </c>
-      <c r="I11" t="s">
-        <v>118</v>
-      </c>
-      <c r="J11" t="s">
-        <v>123</v>
-      </c>
-      <c r="K11" t="s">
-        <v>126</v>
-      </c>
-      <c r="L11" t="s">
-        <v>115</v>
-      </c>
-      <c r="M11" t="s">
-        <v>116</v>
-      </c>
       <c r="N11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="O11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="Q11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -2375,7 +2393,7 @@
         <v>114</v>
       </c>
       <c r="I12" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J12" t="s">
         <v>122</v>
@@ -2390,16 +2408,16 @@
         <v>115</v>
       </c>
       <c r="N12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P12" t="s">
         <v>141</v>
       </c>
       <c r="Q12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -2416,43 +2434,43 @@
         <v>82</v>
       </c>
       <c r="E13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F13" t="s">
         <v>105</v>
       </c>
       <c r="G13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="L13" t="s">
+        <v>115</v>
+      </c>
+      <c r="M13" t="s">
         <v>116</v>
       </c>
-      <c r="M13" t="s">
-        <v>115</v>
-      </c>
       <c r="N13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O13" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P13" t="s">
         <v>140</v>
       </c>
       <c r="Q13" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -2469,43 +2487,43 @@
         <v>83</v>
       </c>
       <c r="E14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F14" t="s">
         <v>106</v>
       </c>
       <c r="G14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H14" t="s">
+        <v>114</v>
+      </c>
+      <c r="I14" t="s">
+        <v>119</v>
+      </c>
+      <c r="J14" t="s">
+        <v>122</v>
+      </c>
+      <c r="K14" t="s">
+        <v>125</v>
+      </c>
+      <c r="L14" t="s">
+        <v>116</v>
+      </c>
+      <c r="M14" t="s">
         <v>115</v>
       </c>
-      <c r="I14" t="s">
-        <v>118</v>
-      </c>
-      <c r="J14" t="s">
-        <v>123</v>
-      </c>
-      <c r="K14" t="s">
-        <v>126</v>
-      </c>
-      <c r="L14" t="s">
-        <v>115</v>
-      </c>
-      <c r="M14" t="s">
-        <v>116</v>
-      </c>
       <c r="N14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="O14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P14" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="Q14" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -2522,22 +2540,22 @@
         <v>84</v>
       </c>
       <c r="E15" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F15" t="s">
         <v>107</v>
       </c>
       <c r="G15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H15" t="s">
         <v>114</v>
       </c>
       <c r="I15" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="J15" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K15" t="s">
         <v>125</v>
@@ -2549,16 +2567,25 @@
         <v>115</v>
       </c>
       <c r="N15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="O15" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="P15" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="Q15" t="s">
-        <v>144</v>
+        <v>151</v>
+      </c>
+      <c r="R15" t="s">
+        <v>154</v>
+      </c>
+      <c r="S15" t="s">
+        <v>158</v>
+      </c>
+      <c r="T15" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -2575,19 +2602,19 @@
         <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F16" t="s">
         <v>108</v>
       </c>
       <c r="G16" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H16" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J16" t="s">
         <v>122</v>
@@ -2599,19 +2626,28 @@
         <v>116</v>
       </c>
       <c r="M16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N16" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="O16" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="P16" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="Q16" t="s">
-        <v>148</v>
+        <v>152</v>
+      </c>
+      <c r="R16" t="s">
+        <v>155</v>
+      </c>
+      <c r="S16" t="s">
+        <v>158</v>
+      </c>
+      <c r="T16" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -2628,52 +2664,52 @@
         <v>86</v>
       </c>
       <c r="E17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F17" t="s">
         <v>109</v>
       </c>
       <c r="G17" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="H17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I17" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K17" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="L17" t="s">
+        <v>115</v>
+      </c>
+      <c r="M17" t="s">
         <v>116</v>
       </c>
-      <c r="M17" t="s">
-        <v>115</v>
-      </c>
       <c r="N17" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P17" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q17" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="R17" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="S17" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="T17" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -2690,19 +2726,19 @@
         <v>87</v>
       </c>
       <c r="E18" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F18" t="s">
         <v>110</v>
       </c>
       <c r="G18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H18" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I18" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J18" t="s">
         <v>122</v>
@@ -2714,28 +2750,28 @@
         <v>116</v>
       </c>
       <c r="M18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="N18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="O18" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="P18" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="Q18" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="R18" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="S18" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="T18" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>